<commit_message>
update Cuentas gestionadas por tony
</commit_message>
<xml_diff>
--- a/gestion.xlsx
+++ b/gestion.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{CCA07C3D-AA16-42B4-8A8F-E56A7C04EEAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBB306ED-E91E-4573-9117-EF9E3056F710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="47">
   <si>
     <t>ID</t>
   </si>
@@ -102,6 +102,66 @@
   </si>
   <si>
     <t>Karla Patiño</t>
+  </si>
+  <si>
+    <t>CRYSTAL GREEN DE MEXICO</t>
+  </si>
+  <si>
+    <t>Seguimiento</t>
+  </si>
+  <si>
+    <t>Se contacta al administrador/ se agenda reunión para presentar a KAM 24/07/2026</t>
+  </si>
+  <si>
+    <t>Jose Antonio Garnica</t>
+  </si>
+  <si>
+    <t>DIVYA</t>
+  </si>
+  <si>
+    <t>En implementación</t>
+  </si>
+  <si>
+    <t>SAMA FOODS</t>
+  </si>
+  <si>
+    <t>Se contacta por telefono a cliente /se agenda reunión hoy día 23/07/26/ SE HACE TRASPASO A KARLA, los clientes quedaron contentos con nuestra atención.</t>
+  </si>
+  <si>
+    <t>ORANGE BUSINESS SERVICES MEXICO</t>
+  </si>
+  <si>
+    <t>Responde Correo electrónico redirigiendo a las personas que podrán atenderme (Esperando se contacten y agenden reunión) 23/07/26</t>
+  </si>
+  <si>
+    <t>VIAJERO HOTELS MX</t>
+  </si>
+  <si>
+    <t>Se envía correo electrónico al administrador 23/06/27</t>
+  </si>
+  <si>
+    <t>VERTIV MEXICO</t>
+  </si>
+  <si>
+    <t>Empresa regional que tiene problemas de momento en México en cuanto a plataforma y quieren implementar alertar en todas las regiones (buscando las reuniones correspondientes) 23/07/26</t>
+  </si>
+  <si>
+    <t>ARAN CONSTRUCCIÓN E INGENIERIA S.A DE C.V (Alves Ribeiro)</t>
+  </si>
+  <si>
+    <t>Se contacta a administradora por telefono, indica que ellos no colocaron ese NPS detractor y que se encuentran muy bien con la atención de KAM KARLA PATIÑO 16/07/26</t>
+  </si>
+  <si>
+    <t>VALIDACION Y METROLOGIA</t>
+  </si>
+  <si>
+    <t>Tenemos reunión el lunes 27 para validar planifiacion y temas en plataforma.</t>
+  </si>
+  <si>
+    <t>HIDALGO VIGUERAS CONSULTORES</t>
+  </si>
+  <si>
+    <t>Se contacta a segundo administrador por telefono 16/07/26, indica que marcan por CALL y que tienen problemas, en espera de que me den fecha para reu. Se manda mensaje de seguimiento sin respuesta (Lunes 20 y hoy 23)</t>
   </si>
   <si>
     <t>Cómo usar este archivo</t>
@@ -609,76 +669,184 @@
       </c>
     </row>
     <row r="3" spans="1:6">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="3"/>
+      <c r="A3" s="2">
+        <v>37535</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="8">
+        <v>46227</v>
+      </c>
     </row>
     <row r="4" spans="1:6">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="3"/>
+      <c r="A4" s="2">
+        <v>38332</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="5" spans="1:6">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="3"/>
+      <c r="A5" s="2">
+        <v>37083</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="F5" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="6" spans="1:6">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="3"/>
+      <c r="A6" s="2">
+        <v>21369</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F6" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="7" spans="1:6">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="3"/>
+      <c r="A7" s="2">
+        <v>35243</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F7" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="8" spans="1:6">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="3"/>
+      <c r="A8" s="2">
+        <v>30860</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="9" spans="1:6">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="3"/>
+      <c r="A9" s="2">
+        <v>35561</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="3">
+        <v>46229</v>
+      </c>
     </row>
     <row r="10" spans="1:6">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="3"/>
+      <c r="A10" s="2">
+        <v>35509</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="11" spans="1:6">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="3"/>
+      <c r="A11" s="2">
+        <v>38089</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F11" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="2"/>
@@ -2213,7 +2381,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -2221,12 +2389,12 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>11</v>
+        <v>31</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="5" t="s">
-        <v>12</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:1">
@@ -2234,37 +2402,37 @@
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="6" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="5" t="s">
-        <v>14</v>
+        <v>34</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="5" t="s">
-        <v>15</v>
+        <v>35</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="5" t="s">
-        <v>16</v>
+        <v>36</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="5" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="5" t="s">
-        <v>18</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="5" t="s">
-        <v>19</v>
+        <v>39</v>
       </c>
     </row>
     <row r="13" spans="1:1">
@@ -2272,27 +2440,27 @@
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="6" t="s">
-        <v>20</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="5" t="s">
-        <v>21</v>
+        <v>41</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="5" t="s">
-        <v>22</v>
+        <v>42</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="5" t="s">
-        <v>23</v>
+        <v>43</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="5" t="s">
-        <v>24</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:1">
@@ -2300,12 +2468,12 @@
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="5" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="5" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update index colores salud y gestion
</commit_message>
<xml_diff>
--- a/gestion.xlsx
+++ b/gestion.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBB306ED-E91E-4573-9117-EF9E3056F710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D5969AA-5C70-4026-97B2-02F21DC49FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="63" uniqueCount="47">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="86">
   <si>
     <t>ID</t>
   </si>
@@ -162,6 +162,123 @@
   </si>
   <si>
     <t>Se contacta a segundo administrador por telefono 16/07/26, indica que marcan por CALL y que tienen problemas, en espera de que me den fecha para reu. Se manda mensaje de seguimiento sin respuesta (Lunes 20 y hoy 23)</t>
+  </si>
+  <si>
+    <t>TRIBUNAL DE JUSTICIA ADMINISTRATIVA DEL ESTADO DE MEXICO (Gobierno del estado de mexico)</t>
+  </si>
+  <si>
+    <t>Están de vacaciones</t>
+  </si>
+  <si>
+    <t>Dafne de la Rosa</t>
+  </si>
+  <si>
+    <t>PIN IT MEDIA</t>
+  </si>
+  <si>
+    <t>SGS DE MEXICO</t>
+  </si>
+  <si>
+    <t>COMERCIALIZADORA IMU</t>
+  </si>
+  <si>
+    <t>PROVEEDOR MAYORISTA AL REFACCIONARIO DE MEXICO</t>
+  </si>
+  <si>
+    <t>TRANSPORTACION Y LOGISTICA MALDONADO</t>
+  </si>
+  <si>
+    <t>GTC TERMO CONTROL</t>
+  </si>
+  <si>
+    <t>GW PLASTICS MEXICANA</t>
+  </si>
+  <si>
+    <t>PLASCENCIA ACUMULADORES</t>
+  </si>
+  <si>
+    <t>METRO ASFALTOS</t>
+  </si>
+  <si>
+    <t>PAN DE PAN MONTERREY</t>
+  </si>
+  <si>
+    <t>ACCORD FARMA</t>
+  </si>
+  <si>
+    <t>CENTROS AUDITIVOS GAES MEXICO</t>
+  </si>
+  <si>
+    <t>ABASTECEDORA AGRICENTER</t>
+  </si>
+  <si>
+    <t>SIERRA NORTE TRUCK CENTER</t>
+  </si>
+  <si>
+    <t>ALCORE INGENIEROS</t>
+  </si>
+  <si>
+    <t>EB SIETE</t>
+  </si>
+  <si>
+    <t>CONSORCIO INDUSTRIAL EDIFICA</t>
+  </si>
+  <si>
+    <t>JUNGLA DE TIMO</t>
+  </si>
+  <si>
+    <t>ARMAZON CONSTRUCTORA</t>
+  </si>
+  <si>
+    <t>LOSEN</t>
+  </si>
+  <si>
+    <t>SOCIEDAD INDUSTRIAL EQUIPOS Y SERVICIOS (SIES)</t>
+  </si>
+  <si>
+    <t>TAGLE BLINDER</t>
+  </si>
+  <si>
+    <t>SERVICIOS ADMINISTRATIVOS TRANSFORMANDO LA EDUCACION DE MEXICO(Innova Schools)</t>
+  </si>
+  <si>
+    <t>Vacaciones</t>
+  </si>
+  <si>
+    <t>Raúl Campos</t>
+  </si>
+  <si>
+    <t>YELTE</t>
+  </si>
+  <si>
+    <t>INSTITUTO TECNOLOGICO SUPERIOR DE ZACAPOAXTLA</t>
+  </si>
+  <si>
+    <t>SCHETTINO</t>
+  </si>
+  <si>
+    <t>SERVIGUE</t>
+  </si>
+  <si>
+    <t>IRKON HOLDINGS</t>
+  </si>
+  <si>
+    <t>Marcaje bajo por piloto</t>
+  </si>
+  <si>
+    <t>TDSYSTEM</t>
+  </si>
+  <si>
+    <t>GRUPO JULIO</t>
+  </si>
+  <si>
+    <t>Tickets resueltos</t>
+  </si>
+  <si>
+    <t>DISTRIBUIDORA JUGUETRON</t>
+  </si>
+  <si>
+    <t>Reunión por NPS ok</t>
   </si>
   <si>
     <t>Cómo usar este archivo</t>
@@ -617,7 +734,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F200"/>
+  <dimension ref="A1:F199"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -849,267 +966,491 @@
       </c>
     </row>
     <row r="12" spans="1:6">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="3"/>
+      <c r="A12" s="2">
+        <v>26820</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F12" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="13" spans="1:6">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
+      <c r="A13" s="2">
+        <v>26820</v>
+      </c>
+      <c r="B13" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="E13" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="F13" s="3"/>
     </row>
     <row r="14" spans="1:6">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
+      <c r="A14" s="2">
+        <v>29825</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>33</v>
+      </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+      <c r="E14" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="F14" s="3"/>
     </row>
     <row r="15" spans="1:6">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
+      <c r="A15" s="2">
+        <v>23418</v>
+      </c>
+      <c r="B15" s="2" t="s">
+        <v>34</v>
+      </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="E15" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="F15" s="3"/>
     </row>
     <row r="16" spans="1:6">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
+      <c r="A16" s="2">
+        <v>21190</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="C16" s="2"/>
       <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="E16" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="F16" s="3"/>
     </row>
     <row r="17" spans="1:6">
-      <c r="A17" s="2"/>
-      <c r="B17" s="2"/>
+      <c r="A17" s="2">
+        <v>21657</v>
+      </c>
+      <c r="B17" s="2" t="s">
+        <v>36</v>
+      </c>
       <c r="C17" s="2"/>
       <c r="D17" s="2"/>
-      <c r="E17" s="2"/>
+      <c r="E17" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="F17" s="3"/>
     </row>
     <row r="18" spans="1:6">
-      <c r="A18" s="2"/>
-      <c r="B18" s="2"/>
+      <c r="A18" s="2">
+        <v>6975</v>
+      </c>
+      <c r="B18" s="2" t="s">
+        <v>37</v>
+      </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+      <c r="E18" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="F18" s="3"/>
     </row>
     <row r="19" spans="1:6">
-      <c r="A19" s="2"/>
-      <c r="B19" s="2"/>
+      <c r="A19" s="2">
+        <v>33503</v>
+      </c>
+      <c r="B19" s="2" t="s">
+        <v>38</v>
+      </c>
       <c r="C19" s="2"/>
       <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
+      <c r="E19" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="F19" s="3"/>
     </row>
     <row r="20" spans="1:6">
-      <c r="A20" s="2"/>
-      <c r="B20" s="2"/>
+      <c r="A20" s="2">
+        <v>24043</v>
+      </c>
+      <c r="B20" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
+      <c r="E20" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F20" s="3"/>
     </row>
     <row r="21" spans="1:6">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
+      <c r="A21" s="2">
+        <v>28896</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>40</v>
+      </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+      <c r="E21" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F21" s="3"/>
     </row>
     <row r="22" spans="1:6">
-      <c r="A22" s="2"/>
-      <c r="B22" s="2"/>
+      <c r="A22" s="2">
+        <v>31808</v>
+      </c>
+      <c r="B22" s="2" t="s">
+        <v>41</v>
+      </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
+      <c r="E22" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F22" s="3"/>
     </row>
     <row r="23" spans="1:6">
-      <c r="A23" s="2"/>
-      <c r="B23" s="2"/>
+      <c r="A23" s="2">
+        <v>17845</v>
+      </c>
+      <c r="B23" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
+      <c r="E23" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F23" s="3"/>
     </row>
     <row r="24" spans="1:6">
-      <c r="A24" s="2"/>
-      <c r="B24" s="2"/>
+      <c r="A24" s="2">
+        <v>26920</v>
+      </c>
+      <c r="B24" s="2" t="s">
+        <v>43</v>
+      </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
-      <c r="E24" s="2"/>
+      <c r="E24" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F24" s="3"/>
     </row>
     <row r="25" spans="1:6">
-      <c r="A25" s="2"/>
-      <c r="B25" s="2"/>
+      <c r="A25" s="2">
+        <v>2418</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
-      <c r="E25" s="2"/>
+      <c r="E25" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F25" s="3"/>
     </row>
     <row r="26" spans="1:6">
-      <c r="A26" s="2"/>
-      <c r="B26" s="2"/>
+      <c r="A26" s="2">
+        <v>26371</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>45</v>
+      </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
-      <c r="E26" s="2"/>
+      <c r="E26" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F26" s="3"/>
     </row>
     <row r="27" spans="1:6">
-      <c r="A27" s="2"/>
-      <c r="B27" s="2"/>
+      <c r="A27" s="2">
+        <v>21436</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
+      <c r="E27" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F27" s="3"/>
     </row>
     <row r="28" spans="1:6">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
+      <c r="A28" s="2">
+        <v>32765</v>
+      </c>
+      <c r="B28" s="2" t="s">
+        <v>47</v>
+      </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
+      <c r="E28" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F28" s="3"/>
     </row>
     <row r="29" spans="1:6">
-      <c r="A29" s="2"/>
-      <c r="B29" s="2"/>
+      <c r="A29" s="2">
+        <v>29844</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>48</v>
+      </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
-      <c r="E29" s="2"/>
+      <c r="E29" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F29" s="3"/>
     </row>
     <row r="30" spans="1:6">
-      <c r="A30" s="2"/>
-      <c r="B30" s="2"/>
+      <c r="A30" s="2">
+        <v>34072</v>
+      </c>
+      <c r="B30" s="2" t="s">
+        <v>49</v>
+      </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
+      <c r="E30" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F30" s="3"/>
     </row>
     <row r="31" spans="1:6">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
+      <c r="A31" s="2">
+        <v>5725</v>
+      </c>
+      <c r="B31" s="2" t="s">
+        <v>50</v>
+      </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
+      <c r="E31" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F31" s="3"/>
     </row>
     <row r="32" spans="1:6">
-      <c r="A32" s="2"/>
-      <c r="B32" s="2"/>
+      <c r="A32" s="2">
+        <v>25626</v>
+      </c>
+      <c r="B32" s="2" t="s">
+        <v>51</v>
+      </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
+      <c r="E32" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F32" s="3"/>
     </row>
     <row r="33" spans="1:6">
-      <c r="A33" s="2"/>
-      <c r="B33" s="2"/>
+      <c r="A33" s="2">
+        <v>6902</v>
+      </c>
+      <c r="B33" s="2" t="s">
+        <v>52</v>
+      </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
+      <c r="E33" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F33" s="3"/>
     </row>
     <row r="34" spans="1:6">
-      <c r="A34" s="2"/>
-      <c r="B34" s="2"/>
+      <c r="A34" s="2">
+        <v>23369</v>
+      </c>
+      <c r="B34" s="2" t="s">
+        <v>53</v>
+      </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
+      <c r="E34" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F34" s="3"/>
     </row>
     <row r="35" spans="1:6">
-      <c r="A35" s="2"/>
-      <c r="B35" s="2"/>
+      <c r="A35" s="2">
+        <v>36040</v>
+      </c>
+      <c r="B35" s="2" t="s">
+        <v>54</v>
+      </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
+      <c r="E35" s="2" t="s">
+        <v>9</v>
+      </c>
       <c r="F35" s="3"/>
     </row>
     <row r="36" spans="1:6">
-      <c r="A36" s="2"/>
-      <c r="B36" s="2"/>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
+      <c r="A36" s="2">
+        <v>20338</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E36" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="F36" s="3"/>
     </row>
     <row r="37" spans="1:6">
-      <c r="A37" s="2"/>
-      <c r="B37" s="2"/>
+      <c r="A37" s="2">
+        <v>24372</v>
+      </c>
+      <c r="B37" s="2" t="s">
+        <v>58</v>
+      </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
+      <c r="E37" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="F37" s="3"/>
     </row>
     <row r="38" spans="1:6">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
+      <c r="A38" s="2">
+        <v>6055</v>
+      </c>
+      <c r="B38" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="F38" s="3"/>
     </row>
     <row r="39" spans="1:6">
-      <c r="A39" s="2"/>
-      <c r="B39" s="2"/>
+      <c r="A39" s="2">
+        <v>6588</v>
+      </c>
+      <c r="B39" s="2" t="s">
+        <v>60</v>
+      </c>
       <c r="C39" s="2"/>
       <c r="D39" s="2"/>
-      <c r="E39" s="2"/>
+      <c r="E39" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="F39" s="3"/>
     </row>
     <row r="40" spans="1:6">
-      <c r="A40" s="2"/>
-      <c r="B40" s="2"/>
+      <c r="A40" s="2">
+        <v>21105</v>
+      </c>
+      <c r="B40" s="2" t="s">
+        <v>61</v>
+      </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
+      <c r="E40" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="F40" s="3"/>
     </row>
     <row r="41" spans="1:6">
-      <c r="A41" s="2"/>
-      <c r="B41" s="2"/>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
+      <c r="A41" s="2">
+        <v>18595</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="C41" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D41" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="F41" s="3"/>
     </row>
     <row r="42" spans="1:6">
-      <c r="A42" s="2"/>
-      <c r="B42" s="2"/>
+      <c r="A42" s="2">
+        <v>24950</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>64</v>
+      </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
+      <c r="E42" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="F42" s="3"/>
     </row>
     <row r="43" spans="1:6">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
+      <c r="A43" s="2">
+        <v>30644</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="E43" s="2" t="s">
+        <v>57</v>
+      </c>
       <c r="F43" s="3"/>
     </row>
     <row r="44" spans="1:6">
-      <c r="A44" s="2"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
+      <c r="A44" s="2">
+        <v>24336</v>
+      </c>
+      <c r="B44" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>68</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>13</v>
+      </c>
       <c r="F44" s="3"/>
     </row>
     <row r="45" spans="1:6">
@@ -2352,17 +2693,9 @@
       <c r="E199" s="2"/>
       <c r="F199" s="3"/>
     </row>
-    <row r="200" spans="1:6">
-      <c r="A200" s="2"/>
-      <c r="B200" s="2"/>
-      <c r="C200" s="2"/>
-      <c r="D200" s="2"/>
-      <c r="E200" s="2"/>
-      <c r="F200" s="3"/>
-    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Estado inválido" error="Elige &quot;Seguimiento&quot; o &quot;Resuelta&quot; de la lista." sqref="C2:C201" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Estado inválido" error="Elige &quot;Seguimiento&quot; o &quot;Resuelta&quot; de la lista." sqref="C2:C200" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Seguimiento,Resuelta"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2381,7 +2714,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>30</v>
+        <v>69</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -2389,12 +2722,12 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>31</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="5" t="s">
-        <v>32</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:1">
@@ -2402,37 +2735,37 @@
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="6" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="5" t="s">
-        <v>34</v>
+        <v>73</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="5" t="s">
-        <v>35</v>
+        <v>74</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="5" t="s">
-        <v>36</v>
+        <v>75</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="5" t="s">
-        <v>37</v>
+        <v>76</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="5" t="s">
-        <v>38</v>
+        <v>77</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="5" t="s">
-        <v>39</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:1">
@@ -2440,27 +2773,27 @@
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="6" t="s">
-        <v>40</v>
+        <v>79</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="5" t="s">
-        <v>41</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="5" t="s">
-        <v>42</v>
+        <v>81</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="5" t="s">
-        <v>43</v>
+        <v>82</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="5" t="s">
-        <v>44</v>
+        <v>83</v>
       </c>
     </row>
     <row r="19" spans="1:1">
@@ -2468,12 +2801,12 @@
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="5" t="s">
-        <v>45</v>
+        <v>84</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="5" t="s">
-        <v>46</v>
+        <v>85</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nueva version de gestion y cartera
</commit_message>
<xml_diff>
--- a/gestion.xlsx
+++ b/gestion.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8D5969AA-5C70-4026-97B2-02F21DC49FEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F3F3979-89A3-4278-84FB-90480B01A14C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="91">
   <si>
     <t>ID</t>
   </si>
@@ -179,18 +179,36 @@
     <t>SGS DE MEXICO</t>
   </si>
   <si>
+    <t>Buscando reunión</t>
+  </si>
+  <si>
     <t>COMERCIALIZADORA IMU</t>
   </si>
   <si>
+    <t>Esperar reu de renovación anualidad para que desactiven usuarios que no están marcando</t>
+  </si>
+  <si>
     <t>PROVEEDOR MAYORISTA AL REFACCIONARIO DE MEXICO</t>
   </si>
   <si>
+    <t>Hubo cambio de admin, seguir monitoreando</t>
+  </si>
+  <si>
     <t>TRANSPORTACION Y LOGISTICA MALDONADO</t>
   </si>
   <si>
     <t>GTC TERMO CONTROL</t>
   </si>
   <si>
+    <t>Esperar nuevo modelo</t>
+  </si>
+  <si>
+    <t>VELEZ CHILDRENS LANGUAGE CENTER</t>
+  </si>
+  <si>
+    <t>Vacaciones</t>
+  </si>
+  <si>
     <t>GW PLASTICS MEXICANA</t>
   </si>
   <si>
@@ -240,9 +258,6 @@
   </si>
   <si>
     <t>SERVICIOS ADMINISTRATIVOS TRANSFORMANDO LA EDUCACION DE MEXICO(Innova Schools)</t>
-  </si>
-  <si>
-    <t>Vacaciones</t>
   </si>
   <si>
     <t>Raúl Campos</t>
@@ -734,7 +749,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F199"/>
+  <dimension ref="A1:F200"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1020,78 +1035,112 @@
       <c r="B15" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
+      <c r="C15" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>35</v>
+      </c>
       <c r="E15" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F15" s="3"/>
+      <c r="F15" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="2">
         <v>21190</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
+        <v>36</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>37</v>
+      </c>
       <c r="E16" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F16" s="3"/>
+      <c r="F16" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="2">
         <v>21657</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="C17" s="2"/>
-      <c r="D17" s="2"/>
+        <v>38</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="E17" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F17" s="3"/>
+      <c r="F17" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="2">
         <v>6975</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
+        <v>40</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>39</v>
+      </c>
       <c r="E18" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F18" s="3"/>
+      <c r="F18" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="2">
         <v>33503</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
+        <v>41</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>42</v>
+      </c>
       <c r="E19" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="F19" s="3"/>
+      <c r="F19" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="2">
-        <v>24043</v>
+        <v>32684</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
+        <v>43</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="E20" s="2" t="s">
         <v>9</v>
       </c>
@@ -1099,10 +1148,10 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="2">
-        <v>28896</v>
+        <v>24043</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="C21" s="2"/>
       <c r="D21" s="2"/>
@@ -1113,10 +1162,10 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="2">
-        <v>31808</v>
+        <v>28896</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -1127,10 +1176,10 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="2">
-        <v>17845</v>
+        <v>31808</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -1141,10 +1190,10 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="2">
-        <v>26920</v>
+        <v>17845</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -1155,10 +1204,10 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="2">
-        <v>2418</v>
+        <v>26920</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -1169,10 +1218,10 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="2">
-        <v>26371</v>
+        <v>2418</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -1183,10 +1232,10 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="2">
-        <v>21436</v>
+        <v>26371</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -1197,10 +1246,10 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="2">
-        <v>32765</v>
+        <v>21436</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -1211,10 +1260,10 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="2">
-        <v>29844</v>
+        <v>32765</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -1225,10 +1274,10 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="2">
-        <v>34072</v>
+        <v>29844</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -1239,10 +1288,10 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="2">
-        <v>5725</v>
+        <v>34072</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -1253,10 +1302,10 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="2">
-        <v>25626</v>
+        <v>5725</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -1267,10 +1316,10 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="2">
-        <v>6902</v>
+        <v>25626</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -1281,10 +1330,10 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="2">
-        <v>23369</v>
+        <v>6902</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -1295,10 +1344,10 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="2">
-        <v>36040</v>
+        <v>23369</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -1309,156 +1358,162 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="2">
-        <v>20338</v>
+        <v>36040</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C36" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D36" s="2" t="s">
-        <v>56</v>
-      </c>
+        <v>60</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
       <c r="E36" s="2" t="s">
-        <v>57</v>
+        <v>9</v>
       </c>
       <c r="F36" s="3"/>
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="2">
-        <v>24372</v>
+        <v>20338</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
+        <v>61</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D37" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="E37" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F37" s="3"/>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="2">
-        <v>6055</v>
+        <v>24372</v>
       </c>
       <c r="B38" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D38" s="2" t="s">
-        <v>56</v>
-      </c>
+        <v>63</v>
+      </c>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
       <c r="E38" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F38" s="3"/>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="2">
-        <v>6588</v>
+        <v>6055</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="C39" s="2"/>
-      <c r="D39" s="2"/>
+        <v>64</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>44</v>
+      </c>
       <c r="E39" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F39" s="3"/>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="2">
-        <v>21105</v>
+        <v>6588</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
       <c r="E40" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F40" s="3"/>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="2">
-        <v>18595</v>
+        <v>21105</v>
       </c>
       <c r="B41" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2" t="s">
         <v>62</v>
-      </c>
-      <c r="C41" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D41" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="E41" s="2" t="s">
-        <v>57</v>
       </c>
       <c r="F41" s="3"/>
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="2">
-        <v>24950</v>
+        <v>18595</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>64</v>
-      </c>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
+        <v>67</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>68</v>
+      </c>
       <c r="E42" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F42" s="3"/>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="2">
-        <v>30644</v>
+        <v>24950</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C43" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D43" s="2" t="s">
-        <v>66</v>
-      </c>
+        <v>69</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
       <c r="E43" s="2" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="F43" s="3"/>
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="2">
-        <v>24336</v>
+        <v>30644</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C44" s="2" t="s">
         <v>7</v>
       </c>
       <c r="D44" s="2" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="E44" s="2" t="s">
+        <v>62</v>
+      </c>
+      <c r="F44" s="3"/>
+    </row>
+    <row r="45" spans="1:6">
+      <c r="A45" s="2">
+        <v>24336</v>
+      </c>
+      <c r="B45" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D45" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="E45" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F44" s="3"/>
-    </row>
-    <row r="45" spans="1:6">
-      <c r="A45" s="2"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
       <c r="F45" s="3"/>
     </row>
     <row r="46" spans="1:6">
@@ -2693,9 +2748,17 @@
       <c r="E199" s="2"/>
       <c r="F199" s="3"/>
     </row>
+    <row r="200" spans="1:6">
+      <c r="A200" s="2"/>
+      <c r="B200" s="2"/>
+      <c r="C200" s="2"/>
+      <c r="D200" s="2"/>
+      <c r="E200" s="2"/>
+      <c r="F200" s="3"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Estado inválido" error="Elige &quot;Seguimiento&quot; o &quot;Resuelta&quot; de la lista." sqref="C2:C200" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Estado inválido" error="Elige &quot;Seguimiento&quot; o &quot;Resuelta&quot; de la lista." sqref="C2:C201" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Seguimiento,Resuelta"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2714,7 +2777,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -2722,12 +2785,12 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="5" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" spans="1:1">
@@ -2735,37 +2798,37 @@
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="6" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="5" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="5" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="5" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="5" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="5" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="5" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
     </row>
     <row r="13" spans="1:1">
@@ -2773,27 +2836,27 @@
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="6" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="5" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="5" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="5" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="5" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
     </row>
     <row r="19" spans="1:1">
@@ -2801,12 +2864,12 @@
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="5" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="5" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
cambio pequeñito en archivos xlsx
</commit_message>
<xml_diff>
--- a/gestion.xlsx
+++ b/gestion.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6F3F3979-89A3-4278-84FB-90480B01A14C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{26B2F635-73D1-4D5A-950D-18501039D0AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -72,7 +72,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="159" uniqueCount="92">
   <si>
     <t>ID</t>
   </si>
@@ -176,6 +176,12 @@
     <t>PIN IT MEDIA</t>
   </si>
   <si>
+    <t>ACTIC</t>
+  </si>
+  <si>
+    <t>Tickets resueltos</t>
+  </si>
+  <si>
     <t>SGS DE MEXICO</t>
   </si>
   <si>
@@ -285,9 +291,6 @@
   </si>
   <si>
     <t>GRUPO JULIO</t>
-  </si>
-  <si>
-    <t>Tickets resueltos</t>
   </si>
   <si>
     <t>DISTRIBUIDORA JUGUETRON</t>
@@ -749,7 +752,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F200"/>
+  <dimension ref="A1:F201"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
@@ -1030,13 +1033,13 @@
     </row>
     <row r="15" spans="1:6">
       <c r="A15" s="2">
-        <v>23418</v>
+        <v>20172</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>34</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>35</v>
@@ -1050,7 +1053,7 @@
     </row>
     <row r="16" spans="1:6">
       <c r="A16" s="2">
-        <v>21190</v>
+        <v>23418</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>36</v>
@@ -1070,7 +1073,7 @@
     </row>
     <row r="17" spans="1:6">
       <c r="A17" s="2">
-        <v>21657</v>
+        <v>21190</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>38</v>
@@ -1090,7 +1093,7 @@
     </row>
     <row r="18" spans="1:6">
       <c r="A18" s="2">
-        <v>6975</v>
+        <v>21657</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>40</v>
@@ -1099,7 +1102,7 @@
         <v>11</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>32</v>
@@ -1110,16 +1113,16 @@
     </row>
     <row r="19" spans="1:6">
       <c r="A19" s="2">
-        <v>33503</v>
+        <v>6975</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C19" s="2" t="s">
         <v>11</v>
       </c>
       <c r="D19" s="2" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>32</v>
@@ -1130,7 +1133,7 @@
     </row>
     <row r="20" spans="1:6">
       <c r="A20" s="2">
-        <v>32684</v>
+        <v>33503</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>43</v>
@@ -1142,19 +1145,25 @@
         <v>44</v>
       </c>
       <c r="E20" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F20" s="3"/>
+        <v>32</v>
+      </c>
+      <c r="F20" s="8">
+        <v>46226</v>
+      </c>
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="2">
-        <v>24043</v>
+        <v>32684</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+      <c r="C21" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="E21" s="2" t="s">
         <v>9</v>
       </c>
@@ -1162,10 +1171,10 @@
     </row>
     <row r="22" spans="1:6">
       <c r="A22" s="2">
-        <v>28896</v>
+        <v>24043</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -1176,10 +1185,10 @@
     </row>
     <row r="23" spans="1:6">
       <c r="A23" s="2">
-        <v>31808</v>
+        <v>28896</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -1190,10 +1199,10 @@
     </row>
     <row r="24" spans="1:6">
       <c r="A24" s="2">
-        <v>17845</v>
+        <v>31808</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
@@ -1204,10 +1213,10 @@
     </row>
     <row r="25" spans="1:6">
       <c r="A25" s="2">
-        <v>26920</v>
+        <v>17845</v>
       </c>
       <c r="B25" s="2" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -1218,10 +1227,10 @@
     </row>
     <row r="26" spans="1:6">
       <c r="A26" s="2">
-        <v>2418</v>
+        <v>26920</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
@@ -1232,10 +1241,10 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="2">
-        <v>26371</v>
+        <v>2418</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -1246,10 +1255,10 @@
     </row>
     <row r="28" spans="1:6">
       <c r="A28" s="2">
-        <v>21436</v>
+        <v>26371</v>
       </c>
       <c r="B28" s="2" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C28" s="2"/>
       <c r="D28" s="2"/>
@@ -1260,10 +1269,10 @@
     </row>
     <row r="29" spans="1:6">
       <c r="A29" s="2">
-        <v>32765</v>
+        <v>21436</v>
       </c>
       <c r="B29" s="2" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C29" s="2"/>
       <c r="D29" s="2"/>
@@ -1274,10 +1283,10 @@
     </row>
     <row r="30" spans="1:6">
       <c r="A30" s="2">
-        <v>29844</v>
+        <v>32765</v>
       </c>
       <c r="B30" s="2" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -1288,10 +1297,10 @@
     </row>
     <row r="31" spans="1:6">
       <c r="A31" s="2">
-        <v>34072</v>
+        <v>29844</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C31" s="2"/>
       <c r="D31" s="2"/>
@@ -1302,10 +1311,10 @@
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="2">
-        <v>5725</v>
+        <v>34072</v>
       </c>
       <c r="B32" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C32" s="2"/>
       <c r="D32" s="2"/>
@@ -1316,10 +1325,10 @@
     </row>
     <row r="33" spans="1:6">
       <c r="A33" s="2">
-        <v>25626</v>
+        <v>5725</v>
       </c>
       <c r="B33" s="2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -1330,10 +1339,10 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="2">
-        <v>6902</v>
+        <v>25626</v>
       </c>
       <c r="B34" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C34" s="2"/>
       <c r="D34" s="2"/>
@@ -1344,10 +1353,10 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="2">
-        <v>23369</v>
+        <v>6902</v>
       </c>
       <c r="B35" s="2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -1358,10 +1367,10 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="2">
-        <v>36040</v>
+        <v>23369</v>
       </c>
       <c r="B36" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -1372,135 +1381,131 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="2">
-        <v>20338</v>
+        <v>36040</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="C37" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D37" s="2" t="s">
-        <v>44</v>
-      </c>
+        <v>62</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
       <c r="E37" s="2" t="s">
-        <v>62</v>
+        <v>9</v>
       </c>
       <c r="F37" s="3"/>
     </row>
     <row r="38" spans="1:6">
       <c r="A38" s="2">
-        <v>24372</v>
+        <v>20338</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
+      <c r="C38" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="E38" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F38" s="3"/>
     </row>
     <row r="39" spans="1:6">
       <c r="A39" s="2">
-        <v>6055</v>
+        <v>24372</v>
       </c>
       <c r="B39" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2" t="s">
         <v>64</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="D39" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="E39" s="2" t="s">
-        <v>62</v>
       </c>
       <c r="F39" s="3"/>
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="2">
-        <v>6588</v>
+        <v>6055</v>
       </c>
       <c r="B40" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
+        <v>66</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D40" s="2" t="s">
+        <v>46</v>
+      </c>
       <c r="E40" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F40" s="3"/>
     </row>
     <row r="41" spans="1:6">
       <c r="A41" s="2">
-        <v>21105</v>
+        <v>6588</v>
       </c>
       <c r="B41" s="2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
       <c r="E41" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F41" s="3"/>
     </row>
     <row r="42" spans="1:6">
       <c r="A42" s="2">
-        <v>18595</v>
+        <v>21105</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>67</v>
-      </c>
-      <c r="C42" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D42" s="2" t="s">
         <v>68</v>
       </c>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
       <c r="E42" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F42" s="3"/>
     </row>
     <row r="43" spans="1:6">
       <c r="A43" s="2">
-        <v>24950</v>
+        <v>18595</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
+      <c r="C43" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>70</v>
+      </c>
       <c r="E43" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F43" s="3"/>
     </row>
     <row r="44" spans="1:6">
       <c r="A44" s="2">
-        <v>30644</v>
+        <v>24950</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="C44" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="D44" s="2" t="s">
         <v>71</v>
       </c>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
       <c r="E44" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F44" s="3"/>
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="2">
-        <v>24336</v>
+        <v>30644</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>72</v>
@@ -1509,19 +1514,29 @@
         <v>7</v>
       </c>
       <c r="D45" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="E45" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="F45" s="3"/>
+    </row>
+    <row r="46" spans="1:6">
+      <c r="A46" s="2">
+        <v>24336</v>
+      </c>
+      <c r="B46" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="E45" s="2" t="s">
+      <c r="C46" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D46" s="2" t="s">
+        <v>74</v>
+      </c>
+      <c r="E46" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F45" s="3"/>
-    </row>
-    <row r="46" spans="1:6">
-      <c r="A46" s="2"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
       <c r="F46" s="3"/>
     </row>
     <row r="47" spans="1:6">
@@ -2756,9 +2771,17 @@
       <c r="E200" s="2"/>
       <c r="F200" s="3"/>
     </row>
+    <row r="201" spans="1:6">
+      <c r="A201" s="2"/>
+      <c r="B201" s="2"/>
+      <c r="C201" s="2"/>
+      <c r="D201" s="2"/>
+      <c r="E201" s="2"/>
+      <c r="F201" s="3"/>
+    </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Estado inválido" error="Elige &quot;Seguimiento&quot; o &quot;Resuelta&quot; de la lista." sqref="C2:C201" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Estado inválido" error="Elige &quot;Seguimiento&quot; o &quot;Resuelta&quot; de la lista." sqref="C2:C202" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Seguimiento,Resuelta"</formula1>
     </dataValidation>
   </dataValidations>
@@ -2777,7 +2800,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -2785,12 +2808,12 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:1">
@@ -2798,37 +2821,37 @@
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="6" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="5" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="5" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="5" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="5" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="5" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="13" spans="1:1">
@@ -2836,27 +2859,27 @@
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="6" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="5" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="5" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="5" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="19" spans="1:1">
@@ -2864,12 +2887,12 @@
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="5" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
nueva version archivo gestion
</commit_message>
<xml_diff>
--- a/gestion.xlsx
+++ b/gestion.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B9BE2AED-9C1C-4828-8952-4DF59E5D9C5F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{8379374C-3134-4452-B070-5E0F03CAE018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -102,6 +102,12 @@
     <t>Razón</t>
   </si>
   <si>
+    <t>MRR</t>
+  </si>
+  <si>
+    <t>N° usuarios</t>
+  </si>
+  <si>
     <t>EXPORTACIONES DIEZ</t>
   </si>
   <si>
@@ -384,25 +390,19 @@
     <t>Implementación</t>
   </si>
   <si>
-    <t>2026-06-22 (7 semanas)</t>
+    <t>Fecha</t>
+  </si>
+  <si>
+    <t>Fecha salud</t>
+  </si>
+  <si>
+    <t>Estado salud</t>
+  </si>
+  <si>
+    <t>CSS</t>
   </si>
   <si>
     <t>Crítico</t>
-  </si>
-  <si>
-    <t>Fecha</t>
-  </si>
-  <si>
-    <t>Fecha salud</t>
-  </si>
-  <si>
-    <t>Estado salud</t>
-  </si>
-  <si>
-    <t>MRR</t>
-  </si>
-  <si>
-    <t>CSS</t>
   </si>
   <si>
     <t>JORGE LEAL SEGOVIA (Fletes Leal)</t>
@@ -977,21 +977,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R169"/>
+  <dimension ref="A1:R163"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
     <col min="4" max="4" width="14" customWidth="1"/>
-    <col min="5" max="5" width="188.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="87.42578125" customWidth="1"/>
     <col min="6" max="6" width="21.28515625" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="17.42578125" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="11.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="20.100000000000001" customHeight="1">
+    <row r="1" spans="1:10" ht="20.100000000000001" customHeight="1">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1016,8 +1016,14 @@
       <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" s="16">
         <v>46223</v>
       </c>
@@ -1025,23 +1031,23 @@
         <v>36134</v>
       </c>
       <c r="C2" s="24" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D2" s="24" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E2" s="24" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F2" s="24" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G2" s="24" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H2" s="17"/>
     </row>
-    <row r="3" spans="1:8">
+    <row r="3" spans="1:10">
       <c r="A3" s="11">
         <v>46227</v>
       </c>
@@ -1049,23 +1055,23 @@
         <v>37535</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H3" s="12"/>
     </row>
-    <row r="4" spans="1:8">
+    <row r="4" spans="1:10">
       <c r="A4" s="11">
         <v>46226</v>
       </c>
@@ -1073,25 +1079,25 @@
         <v>38332</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E4" s="10" t="s">
+        <v>19</v>
+      </c>
+      <c r="F4" s="10" t="s">
+        <v>13</v>
+      </c>
+      <c r="G4" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="F4" s="10" t="s">
-        <v>11</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>15</v>
-      </c>
       <c r="H4" s="12" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" s="17" customFormat="1">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" s="17" customFormat="1">
       <c r="A5" s="16">
         <v>46226</v>
       </c>
@@ -1099,22 +1105,22 @@
         <v>37083</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D5" s="15" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E5" s="15" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="F5" s="15" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G5" s="15" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
       <c r="A6" s="13">
         <v>46226</v>
       </c>
@@ -1122,23 +1128,23 @@
         <v>21369</v>
       </c>
       <c r="C6" s="9" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D6" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E6" s="9" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="F6" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G6" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H6" s="14"/>
     </row>
-    <row r="7" spans="1:8">
+    <row r="7" spans="1:10">
       <c r="A7" s="16">
         <v>46226</v>
       </c>
@@ -1146,23 +1152,23 @@
         <v>30860</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D7" s="15" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E7" s="15" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F7" s="15" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G7" s="15" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H7" s="17"/>
     </row>
-    <row r="8" spans="1:8">
+    <row r="8" spans="1:10">
       <c r="A8" s="18">
         <v>46229</v>
       </c>
@@ -1170,23 +1176,23 @@
         <v>35561</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="D8" s="15" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E8" s="15" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="F8" s="15" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G8" s="15" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H8" s="17"/>
     </row>
-    <row r="9" spans="1:8" s="17" customFormat="1" ht="43.5">
+    <row r="9" spans="1:10" s="17" customFormat="1" ht="43.5">
       <c r="A9" s="16">
         <v>46226</v>
       </c>
@@ -1194,25 +1200,25 @@
         <v>35509</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D9" s="15" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E9" s="30" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F9" s="31" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G9" s="15" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H9" s="17" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="43.5">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" ht="43.5">
       <c r="A10" s="13">
         <v>46226</v>
       </c>
@@ -1220,25 +1226,25 @@
         <v>38089</v>
       </c>
       <c r="C10" s="9" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E10" s="19" t="s">
+        <v>33</v>
+      </c>
+      <c r="F10" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="G10" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H10" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="F10" s="19" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="H10" s="14" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
+    </row>
+    <row r="11" spans="1:10">
       <c r="A11" s="26">
         <v>46226</v>
       </c>
@@ -1246,43 +1252,43 @@
         <v>26820</v>
       </c>
       <c r="C11" s="25" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="D11" s="25" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E11" s="25" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F11" s="25" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G11" s="25" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H11" s="27"/>
     </row>
-    <row r="12" spans="1:8">
+    <row r="12" spans="1:10">
       <c r="A12" s="3"/>
       <c r="B12" s="2">
         <v>29825</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
       <c r="F12" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G12" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H12" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10">
       <c r="A13" s="16">
         <v>46226</v>
       </c>
@@ -1290,23 +1296,23 @@
         <v>20172</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="D13" s="15" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E13" s="15" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F13" s="15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G13" s="15" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="H13" s="17"/>
     </row>
-    <row r="14" spans="1:8">
+    <row r="14" spans="1:10">
       <c r="A14" s="13">
         <v>46226</v>
       </c>
@@ -1314,25 +1320,25 @@
         <v>23418</v>
       </c>
       <c r="C14" s="9" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E14" s="9" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="F14" s="9" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H14" s="14" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
       <c r="A15" s="7">
         <v>46226</v>
       </c>
@@ -1340,22 +1346,22 @@
         <v>21190</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D15" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="F15" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G15" s="2" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
       <c r="A16" s="7">
         <v>46226</v>
       </c>
@@ -1363,19 +1369,19 @@
         <v>21657</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F16" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G16" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" spans="1:18">
@@ -1386,19 +1392,19 @@
         <v>6975</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D17" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F17" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="18" spans="1:18">
@@ -1409,19 +1415,19 @@
         <v>33503</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="D18" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E18" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="F18" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G18" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
     </row>
     <row r="19" spans="1:18">
@@ -1430,19 +1436,19 @@
         <v>32684</v>
       </c>
       <c r="C19" s="25" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D19" s="25" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E19" s="25" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F19" s="25" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G19" s="25" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H19" s="27"/>
     </row>
@@ -1452,19 +1458,19 @@
         <v>24043</v>
       </c>
       <c r="C20" s="9" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F20" s="9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H20" s="38">
         <v>0.33</v>
@@ -1477,19 +1483,19 @@
         <v>28896</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E21" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="F21" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H21" s="29">
         <v>0.05</v>
@@ -1502,19 +1508,19 @@
         <v>31808</v>
       </c>
       <c r="C22" s="33" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="D22" s="33" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="F22" s="33" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G22" s="33" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H22" s="35">
         <v>0.25</v>
@@ -1527,19 +1533,19 @@
         <v>26920</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D23" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E23" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F23" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="R23" s="8"/>
     </row>
@@ -1549,19 +1555,19 @@
         <v>2418</v>
       </c>
       <c r="C24" s="33" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D24" s="33" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F24" s="33" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G24" s="33" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H24" s="35">
         <v>0.52</v>
@@ -1575,19 +1581,19 @@
         <v>26371</v>
       </c>
       <c r="C25" s="33" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="D25" s="33" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E25" s="33" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="F25" s="33" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G25" s="33" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H25" s="35">
         <v>0.55000000000000004</v>
@@ -1600,19 +1606,19 @@
         <v>21436</v>
       </c>
       <c r="C26" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="D26" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E26" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="F26" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G26" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="Q26" s="8"/>
       <c r="R26" s="8"/>
@@ -1623,20 +1629,20 @@
         <v>5725</v>
       </c>
       <c r="C27" s="21" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="D27" s="21"/>
       <c r="E27" s="21" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F27" s="21" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G27" s="21" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="H27" s="23" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="R27" s="8"/>
     </row>
@@ -1646,22 +1652,22 @@
         <v>25626</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D28" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E28" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F28" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G28" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H28" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="Q28" s="8"/>
       <c r="R28" s="8"/>
@@ -1672,19 +1678,19 @@
         <v>20338</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D29" s="25" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E29" s="25" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F29" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G29" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H29" s="27"/>
       <c r="R29" s="8"/>
@@ -1695,18 +1701,18 @@
         <v>24372</v>
       </c>
       <c r="C30" s="33" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D30" s="33"/>
       <c r="E30" s="33"/>
       <c r="F30" s="33" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G30" s="33" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H30" s="36" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="Q30" s="37"/>
       <c r="R30" s="37"/>
@@ -1717,19 +1723,19 @@
         <v>6055</v>
       </c>
       <c r="C31" s="25" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D31" s="25" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E31" s="25" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="F31" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G31" s="25" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H31" s="27"/>
       <c r="R31" s="8"/>
@@ -1740,15 +1746,15 @@
         <v>6588</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G32" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H32" s="29">
         <v>0.42</v>
@@ -1762,15 +1768,15 @@
         <v>21105</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D33" s="2"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G33" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H33" s="29">
         <v>0.44</v>
@@ -1783,19 +1789,19 @@
         <v>18595</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D34" s="15" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="F34" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="H34" s="17"/>
       <c r="Q34" s="8"/>
@@ -1807,19 +1813,19 @@
         <v>24950</v>
       </c>
       <c r="C35" s="9" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="F35" s="9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="Q35" s="32"/>
       <c r="R35" s="32"/>
@@ -1830,19 +1836,19 @@
         <v>30644</v>
       </c>
       <c r="C36" s="15" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="D36" s="15" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E36" s="15" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="F36" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G36" s="15" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H36" s="17"/>
       <c r="R36" s="8"/>
@@ -1853,19 +1859,19 @@
         <v>24336</v>
       </c>
       <c r="C37" s="15" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="D37" s="15" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E37" s="15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F37" s="15" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="G37" s="15" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H37" s="17"/>
       <c r="Q37" s="8"/>
@@ -1877,20 +1883,20 @@
         <v>30029</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="D38" s="2"/>
       <c r="E38" s="2" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="F38" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G38" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H38" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="R38" s="8"/>
     </row>
@@ -1900,20 +1906,20 @@
         <v>33301</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="D39" s="2"/>
       <c r="E39" s="2" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="F39" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G39" s="2" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H39" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="R39" s="8"/>
     </row>
@@ -1923,48 +1929,42 @@
         <v>20442</v>
       </c>
       <c r="C40" s="2" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D40" s="2" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="E40" s="2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F40" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G40" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H40" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="R40" s="8"/>
     </row>
     <row r="41" spans="1:18">
       <c r="A41" s="3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B41" s="2"/>
       <c r="C41" s="2" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="E41" s="2"/>
       <c r="F41" s="2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>11</v>
-      </c>
-      <c r="I41" t="s">
-        <v>96</v>
-      </c>
-      <c r="J41" t="s">
-        <v>97</v>
+        <v>13</v>
       </c>
       <c r="K41">
         <v>188</v>
@@ -1981,8 +1981,6 @@
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
       <c r="G42" s="2"/>
-      <c r="Q42" s="8"/>
-      <c r="R42" s="8"/>
     </row>
     <row r="43" spans="1:18">
       <c r="A43" s="3"/>
@@ -1992,7 +1990,6 @@
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
-      <c r="R43" s="8"/>
     </row>
     <row r="44" spans="1:18">
       <c r="A44" s="3"/>
@@ -2002,8 +1999,15 @@
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
-      <c r="Q44" s="8"/>
-      <c r="R44" s="8"/>
+    </row>
+    <row r="45" spans="1:18">
+      <c r="A45" s="3"/>
+      <c r="B45" s="2"/>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+      <c r="G45" s="2"/>
     </row>
     <row r="46" spans="1:18">
       <c r="A46" s="3"/>
@@ -3067,64 +3071,10 @@
       <c r="F163" s="2"/>
       <c r="G163" s="2"/>
     </row>
-    <row r="164" spans="1:7">
-      <c r="A164" s="3"/>
-      <c r="B164" s="2"/>
-      <c r="C164" s="2"/>
-      <c r="D164" s="2"/>
-      <c r="E164" s="2"/>
-      <c r="F164" s="2"/>
-      <c r="G164" s="2"/>
-    </row>
-    <row r="165" spans="1:7">
-      <c r="A165" s="3"/>
-      <c r="B165" s="2"/>
-      <c r="C165" s="2"/>
-      <c r="D165" s="2"/>
-      <c r="E165" s="2"/>
-      <c r="F165" s="2"/>
-      <c r="G165" s="2"/>
-    </row>
-    <row r="166" spans="1:7">
-      <c r="A166" s="3"/>
-      <c r="B166" s="2"/>
-      <c r="C166" s="2"/>
-      <c r="D166" s="2"/>
-      <c r="E166" s="2"/>
-      <c r="F166" s="2"/>
-      <c r="G166" s="2"/>
-    </row>
-    <row r="167" spans="1:7">
-      <c r="A167" s="3"/>
-      <c r="B167" s="2"/>
-      <c r="C167" s="2"/>
-      <c r="D167" s="2"/>
-      <c r="E167" s="2"/>
-      <c r="F167" s="2"/>
-      <c r="G167" s="2"/>
-    </row>
-    <row r="168" spans="1:7">
-      <c r="A168" s="3"/>
-      <c r="B168" s="2"/>
-      <c r="C168" s="2"/>
-      <c r="D168" s="2"/>
-      <c r="E168" s="2"/>
-      <c r="F168" s="2"/>
-      <c r="G168" s="2"/>
-    </row>
-    <row r="169" spans="1:7">
-      <c r="A169" s="3"/>
-      <c r="B169" s="2"/>
-      <c r="C169" s="2"/>
-      <c r="D169" s="2"/>
-      <c r="E169" s="2"/>
-      <c r="F169" s="2"/>
-      <c r="G169" s="2"/>
-    </row>
   </sheetData>
   <autoFilter ref="B1:G40" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Estado inválido" error="Elige &quot;Seguimiento&quot; o &quot;Resuelta&quot; de la lista." sqref="D2:D44 A46:A170 D46:D170 A2:A44" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Estado inválido" error="Elige &quot;Seguimiento&quot; o &quot;Resuelta&quot; de la lista." sqref="D2:D164 A2:A164" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Seguimiento,Resuelta"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3164,10 +3114,10 @@
         <v>100</v>
       </c>
       <c r="Q8" t="s">
+        <v>8</v>
+      </c>
+      <c r="R8" t="s">
         <v>101</v>
-      </c>
-      <c r="R8" t="s">
-        <v>102</v>
       </c>
     </row>
     <row r="9" spans="9:18">
@@ -3175,16 +3125,16 @@
         <v>2418</v>
       </c>
       <c r="J9" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="M9" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O9" s="8">
         <v>46230</v>
       </c>
       <c r="P9" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q9">
         <v>89</v>
@@ -3195,16 +3145,16 @@
         <v>28896</v>
       </c>
       <c r="J10" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="M10" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O10" s="8">
         <v>46230</v>
       </c>
       <c r="P10" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q10">
         <v>109</v>
@@ -3215,16 +3165,16 @@
         <v>25626</v>
       </c>
       <c r="J11" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="M11" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O11" s="8">
         <v>46230</v>
       </c>
       <c r="P11" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q11">
         <v>117</v>
@@ -3235,16 +3185,16 @@
         <v>26371</v>
       </c>
       <c r="J12" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="M12" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O12" s="8">
         <v>46230</v>
       </c>
       <c r="P12" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q12">
         <v>140</v>
@@ -3258,13 +3208,13 @@
         <v>103</v>
       </c>
       <c r="M13" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O13" s="8">
         <v>46230</v>
       </c>
       <c r="P13" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q13">
         <v>161</v>
@@ -3275,16 +3225,16 @@
         <v>36134</v>
       </c>
       <c r="J14" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="K14" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L14" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="M14" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N14" s="8">
         <v>46223</v>
@@ -3293,7 +3243,7 @@
         <v>46230</v>
       </c>
       <c r="P14" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q14">
         <v>171</v>
@@ -3304,16 +3254,16 @@
         <v>26920</v>
       </c>
       <c r="J15" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="M15" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O15" s="8">
         <v>46230</v>
       </c>
       <c r="P15" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q15">
         <v>188</v>
@@ -3324,16 +3274,16 @@
         <v>35561</v>
       </c>
       <c r="J16" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="K16" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L16" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="M16" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N16" s="8">
         <v>46229</v>
@@ -3342,7 +3292,7 @@
         <v>46230</v>
       </c>
       <c r="P16" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q16">
         <v>220</v>
@@ -3353,16 +3303,16 @@
         <v>24043</v>
       </c>
       <c r="J17" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="M17" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O17" s="8">
         <v>46230</v>
       </c>
       <c r="P17" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q17">
         <v>273</v>
@@ -3373,16 +3323,16 @@
         <v>31808</v>
       </c>
       <c r="J18" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="M18" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O18" s="8">
         <v>46230</v>
       </c>
       <c r="P18" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q18">
         <v>375</v>
@@ -3393,16 +3343,16 @@
         <v>21436</v>
       </c>
       <c r="J19" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="M19" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O19" s="8">
         <v>46230</v>
       </c>
       <c r="P19" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q19">
         <v>435</v>
@@ -3413,16 +3363,16 @@
         <v>5725</v>
       </c>
       <c r="J20" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="M20" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O20" s="8">
         <v>46230</v>
       </c>
       <c r="P20" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q20">
         <v>156</v>
@@ -3433,16 +3383,16 @@
         <v>21369</v>
       </c>
       <c r="J21" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K21" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L21" t="s">
         <v>104</v>
       </c>
       <c r="M21" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N21" s="8">
         <v>46226</v>
@@ -3451,7 +3401,7 @@
         <v>46230</v>
       </c>
       <c r="P21" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q21">
         <v>156</v>
@@ -3462,16 +3412,16 @@
         <v>33301</v>
       </c>
       <c r="J22" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="M22" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O22" s="8">
         <v>46230</v>
       </c>
       <c r="P22" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q22">
         <v>165</v>
@@ -3482,22 +3432,22 @@
         <v>32684</v>
       </c>
       <c r="J23" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="K23" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L23" t="s">
         <v>105</v>
       </c>
       <c r="M23" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O23" s="8">
         <v>46230</v>
       </c>
       <c r="P23" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q23">
         <v>166</v>
@@ -3511,13 +3461,13 @@
         <v>106</v>
       </c>
       <c r="M24" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O24" s="8">
         <v>46230</v>
       </c>
       <c r="P24" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q24">
         <v>187</v>
@@ -3525,16 +3475,16 @@
     </row>
     <row r="25" spans="9:17">
       <c r="J25" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="M25" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O25" s="8">
         <v>46230</v>
       </c>
       <c r="P25" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q25">
         <v>188</v>
@@ -3545,16 +3495,16 @@
         <v>35509</v>
       </c>
       <c r="J26" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="K26" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L26" t="s">
         <v>107</v>
       </c>
       <c r="M26" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N26" s="8">
         <v>46226</v>
@@ -3563,7 +3513,7 @@
         <v>46230</v>
       </c>
       <c r="P26" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q26">
         <v>189</v>
@@ -3577,13 +3527,13 @@
         <v>108</v>
       </c>
       <c r="M27" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O27" s="8">
         <v>46230</v>
       </c>
       <c r="P27" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q27">
         <v>270</v>
@@ -3591,16 +3541,16 @@
     </row>
     <row r="28" spans="9:17">
       <c r="J28" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K28" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L28" t="s">
+        <v>19</v>
+      </c>
+      <c r="M28" t="s">
         <v>17</v>
-      </c>
-      <c r="M28" t="s">
-        <v>15</v>
       </c>
       <c r="N28" s="8">
         <v>46226</v>
@@ -3609,7 +3559,7 @@
         <v>46230</v>
       </c>
       <c r="P28" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q28">
         <v>290</v>
@@ -3620,13 +3570,13 @@
         <v>109</v>
       </c>
       <c r="M29" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O29" s="8">
         <v>46230</v>
       </c>
       <c r="P29" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q29">
         <v>303</v>
@@ -3637,16 +3587,16 @@
         <v>30860</v>
       </c>
       <c r="J30" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="K30" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="L30" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="M30" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N30" s="8">
         <v>46226</v>
@@ -3655,7 +3605,7 @@
         <v>46230</v>
       </c>
       <c r="P30" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q30">
         <v>310</v>
@@ -3663,16 +3613,16 @@
     </row>
     <row r="31" spans="9:17">
       <c r="J31" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="K31" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L31" t="s">
         <v>110</v>
       </c>
       <c r="M31" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="N31" s="8">
         <v>46226</v>
@@ -3681,7 +3631,7 @@
         <v>46230</v>
       </c>
       <c r="P31" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="Q31">
         <v>423</v>
@@ -3695,7 +3645,7 @@
         <v>111</v>
       </c>
       <c r="M32" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O32" s="8">
         <v>46230</v>
@@ -3712,16 +3662,16 @@
         <v>37083</v>
       </c>
       <c r="J33" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K33" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="L33" t="s">
         <v>113</v>
       </c>
       <c r="M33" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N33" s="8">
         <v>46226</v>
@@ -3744,7 +3694,7 @@
         <v>114</v>
       </c>
       <c r="M34" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="O34" s="8">
         <v>46230</v>

</xml_diff>

<commit_message>
nueva version cartera, gestion
</commit_message>
<xml_diff>
--- a/gestion.xlsx
+++ b/gestion.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{8379374C-3134-4452-B070-5E0F03CAE018}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{1A2144BC-E1CD-4A0E-B618-A73F8CA3263A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -13,7 +13,7 @@
     <sheet name="Instrucciones" sheetId="2" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Gestión!$B$1:$G$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Gestión!$B$1:$G$37</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -76,7 +76,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="132">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="162">
   <si>
     <t>Fecha Salud</t>
   </si>
@@ -207,187 +207,283 @@
     <t>Dafne de la Rosa</t>
   </si>
   <si>
+    <t>ACTIC</t>
+  </si>
+  <si>
+    <t>Tickets resueltos</t>
+  </si>
+  <si>
+    <t>SGS DE MEXICO</t>
+  </si>
+  <si>
+    <t>Buscando reunión</t>
+  </si>
+  <si>
+    <t>Marcaje 21%</t>
+  </si>
+  <si>
+    <t>COMERCIALIZADORA IMU</t>
+  </si>
+  <si>
+    <t>Esperar reu de renovación anualidad para que desactiven usuarios que no están marcando</t>
+  </si>
+  <si>
+    <t>PROVEEDOR MAYORISTA AL REFACCIONARIO DE MEXICO</t>
+  </si>
+  <si>
+    <t>Hubo cambio de admin, seguir monitoreando</t>
+  </si>
+  <si>
+    <t>TRANSPORTACION Y LOGISTICA MALDONADO</t>
+  </si>
+  <si>
+    <t>GTC TERMO CONTROL</t>
+  </si>
+  <si>
+    <t>Esperar nuevo modelo</t>
+  </si>
+  <si>
+    <t>VELEZ CHILDRENS LANGUAGE CENTER</t>
+  </si>
+  <si>
+    <t>GW PLASTICS MEXICANA</t>
+  </si>
+  <si>
+    <t>Sin respuesta, pasar contacto a Tony/ Se envia mensaje por whatsApp 10/08/2026</t>
+  </si>
+  <si>
+    <t>PLASCENCIA ACUMULADORES</t>
+  </si>
+  <si>
+    <t>Fallaba reloj, ya está ok. Revisar salud proxima semana. Sigue en 5%, volver a revisar</t>
+  </si>
+  <si>
+    <t>METRO ASFALTOS</t>
+  </si>
+  <si>
+    <t>Sin respuesta, pasar contacto a Tony</t>
+  </si>
+  <si>
+    <t>ACCORD FARMA</t>
+  </si>
+  <si>
+    <t>Tuvieron que mover biometrico, revisar salud de proxima semana, ya deberían estar ok</t>
+  </si>
+  <si>
+    <t>CENTROS AUDITIVOS GAES MEXICO</t>
+  </si>
+  <si>
+    <t>Se contactó al cliente, no ve nada raro. Ver segumiento. Tony revisar listado de usuarios que no están marcados</t>
+  </si>
+  <si>
+    <t>ABASTECEDORA AGRICENTER</t>
+  </si>
+  <si>
+    <t>Revisando marcajes de parte de cliente. Tony sacar listado de colaboradores que no marcan</t>
+  </si>
+  <si>
+    <t>SIERRA NORTE TRUCK CENTER</t>
+  </si>
+  <si>
+    <t>Usuarios no tenían correos, no pueden entrar. Esperando correos</t>
+  </si>
+  <si>
+    <t>2026-06-22 (8 semanas)</t>
+  </si>
+  <si>
+    <t>JUNGLA DE TIMO</t>
+  </si>
+  <si>
+    <t>Pendiente reu con el partner</t>
+  </si>
+  <si>
+    <t>Fernanda Durán</t>
+  </si>
+  <si>
+    <t>Marcaje 81% - NPS 0 - Tickets 0</t>
+  </si>
+  <si>
+    <t>ARMAZON CONSTRUCTORA</t>
+  </si>
+  <si>
+    <t>Muchas dudas, pero no tiene mayores complicaciones. Comunicación por correo</t>
+  </si>
+  <si>
+    <t>SERVICIOS ADMINISTRATIVOS TRANSFORMANDO LA EDUCACION DE MEXICO(Innova Schools)</t>
+  </si>
+  <si>
+    <t>Raúl Campos</t>
+  </si>
+  <si>
+    <t>INSTITUTO TECNOLOGICO SUPERIOR DE ZACAPOAXTLA</t>
+  </si>
+  <si>
+    <t>SERVIGUE</t>
+  </si>
+  <si>
+    <t>Repuntó - 10 de agosto marcando 78%</t>
+  </si>
+  <si>
+    <t>IRKON HOLDINGS</t>
+  </si>
+  <si>
+    <t>Marcaje bajo por piloto</t>
+  </si>
+  <si>
+    <t>TDSYSTEM</t>
+  </si>
+  <si>
+    <t>Me contacto con el administrado por medio de llamada, indica que se va de vacaciones dos semanas y que el bajo marcaje es por una renuencia de los colaboradores, adicional quieren validar temas de vaciones regresando, no se arma aún reunión. 31/07/26</t>
+  </si>
+  <si>
+    <t>GRUPO JULIO</t>
+  </si>
+  <si>
+    <t>Tickets resueltos. Son por desconexión de reloj, pero pasa por bajas de voltaje en sus sucursales</t>
+  </si>
+  <si>
+    <t>DISTRIBUIDORA JUGUETRON</t>
+  </si>
+  <si>
+    <t>Reunión por NPS ok</t>
+  </si>
+  <si>
+    <t>2026-08-10 (1 semana)</t>
+  </si>
+  <si>
+    <t>INTEGRITY PROTECTION SERVICES (IPS)</t>
+  </si>
+  <si>
+    <t>No ha habido respuesta</t>
+  </si>
+  <si>
+    <t>Marcaje 27% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>NSF DE MEXICO</t>
+  </si>
+  <si>
+    <t>Sin contacto</t>
+  </si>
+  <si>
+    <t>Marcaje 31% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>Fletes Leal</t>
+  </si>
+  <si>
+    <t>Ver si además bajo marcaje sirve para vender alertas/ Tuve llamada con esta empresa, el marcaje bajo se debe a que sus coalaboradores no llegan a sitio donde se encuentra reloj para marcar y con Karla ya estan implementando APP, tendre reunión con ellos el día 14 de Agosto para dudas en plataforma.</t>
+  </si>
+  <si>
+    <t>Marcaje 50%</t>
+  </si>
+  <si>
+    <t>HEXAGON MINING MEXICO</t>
+  </si>
+  <si>
+    <t>Marcaje 26% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>2026-07-27 (3 semanas)</t>
+  </si>
+  <si>
+    <t>SCHETTINO</t>
+  </si>
+  <si>
+    <t>Marcaje 43% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>AJEMEX</t>
+  </si>
+  <si>
+    <t>3 tickets incidencias de reloj desconectado, ya fueron solucionados</t>
+  </si>
+  <si>
+    <t>Marcaje 79% - NPS s/d - Tickets 3</t>
+  </si>
+  <si>
+    <t>38149-24834</t>
+  </si>
+  <si>
+    <t>FIDES SEGURIDAD PRIVADA</t>
+  </si>
+  <si>
+    <t>Marcaje 2% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>YELTE</t>
+  </si>
+  <si>
+    <t>Acompañamiento - Marcaje 12% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>PORCELANA CORONA DE MEXICO, SA. CV.</t>
+  </si>
+  <si>
+    <t>Marcaje 40% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>2026-08-03 (2 semanas)</t>
+  </si>
+  <si>
+    <t>TAKE FLIGHT VENTURES</t>
+  </si>
+  <si>
+    <t>Marcaje 83% - NPS s/d - Tickets 3</t>
+  </si>
+  <si>
+    <t>OVERHAUL RISK MANAGEMENT</t>
+  </si>
+  <si>
+    <t>Marcaje 59% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>ISEG MEXICO SEGURIDAD PRIVADA</t>
+  </si>
+  <si>
+    <t>Marcaje 47% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>LOGICAMEX</t>
+  </si>
+  <si>
+    <t>Marcaje 2% - NPS s/d - Tickets 1</t>
+  </si>
+  <si>
     <t>PIN IT MEDIA</t>
   </si>
   <si>
-    <t>Acompañamiento.</t>
-  </si>
-  <si>
-    <t>ACTIC</t>
-  </si>
-  <si>
-    <t>Tickets resueltos</t>
-  </si>
-  <si>
-    <t>SGS DE MEXICO</t>
-  </si>
-  <si>
-    <t>Buscando reunión</t>
-  </si>
-  <si>
-    <t>Marcaje 21%</t>
-  </si>
-  <si>
-    <t>COMERCIALIZADORA IMU</t>
-  </si>
-  <si>
-    <t>Esperar reu de renovación anualidad para que desactiven usuarios que no están marcando</t>
-  </si>
-  <si>
-    <t>PROVEEDOR MAYORISTA AL REFACCIONARIO DE MEXICO</t>
-  </si>
-  <si>
-    <t>Hubo cambio de admin, seguir monitoreando</t>
-  </si>
-  <si>
-    <t>TRANSPORTACION Y LOGISTICA MALDONADO</t>
-  </si>
-  <si>
-    <t>GTC TERMO CONTROL</t>
-  </si>
-  <si>
-    <t>Esperar nuevo modelo</t>
-  </si>
-  <si>
-    <t>VELEZ CHILDRENS LANGUAGE CENTER</t>
-  </si>
-  <si>
-    <t>GW PLASTICS MEXICANA</t>
-  </si>
-  <si>
-    <t>Sin respuesta, pasar contacto a Tony/ Se envia mensaje por whatsApp 10/08/2026</t>
-  </si>
-  <si>
-    <t>PLASCENCIA ACUMULADORES</t>
-  </si>
-  <si>
-    <t>Fallaba reloj, ya está ok. Revisar salud proxima semana. Sigue en 5%, volver a revisar</t>
-  </si>
-  <si>
-    <t>METRO ASFALTOS</t>
-  </si>
-  <si>
-    <t>Sin respuesta, pasar contacto a Tony</t>
-  </si>
-  <si>
-    <t>ACCORD FARMA</t>
-  </si>
-  <si>
-    <t>Tuvieron que mover biometrico, revisar salud de proxima semana, ya deberían estar ok</t>
-  </si>
-  <si>
-    <t>CENTROS AUDITIVOS GAES MEXICO</t>
-  </si>
-  <si>
-    <t>Se contactó al cliente, no ve nada raro. Ver segumiento. Tony revisar listado de usuarios que no están marcados</t>
-  </si>
-  <si>
-    <t>ABASTECEDORA AGRICENTER</t>
-  </si>
-  <si>
-    <t>Revisando marcajes de parte de cliente. Tony sacar listado de colaboradores que no marcan</t>
-  </si>
-  <si>
-    <t>SIERRA NORTE TRUCK CENTER</t>
-  </si>
-  <si>
-    <t>Usuarios no tenían correos, no pueden entrar. Esperando correos</t>
-  </si>
-  <si>
-    <t>JUNGLA DE TIMO</t>
-  </si>
-  <si>
-    <t>Pendiente reu con el partner</t>
-  </si>
-  <si>
-    <t>Fernanda Durán</t>
-  </si>
-  <si>
-    <t>ARMAZON CONSTRUCTORA</t>
-  </si>
-  <si>
-    <t>Muchas dudas, pero no tiene mayores complicaciones. Comunicación por correo</t>
-  </si>
-  <si>
-    <t>SERVICIOS ADMINISTRATIVOS TRANSFORMANDO LA EDUCACION DE MEXICO(Innova Schools)</t>
-  </si>
-  <si>
-    <t>Raúl Campos</t>
-  </si>
-  <si>
-    <t>YELTE</t>
-  </si>
-  <si>
-    <t>Acompañmiento (23%)</t>
-  </si>
-  <si>
-    <t>INSTITUTO TECNOLOGICO SUPERIOR DE ZACAPOAXTLA</t>
-  </si>
-  <si>
-    <t>SCHETTINO</t>
-  </si>
-  <si>
-    <t>SERVIGUE</t>
-  </si>
-  <si>
-    <t>IRKON HOLDINGS</t>
-  </si>
-  <si>
-    <t>Marcaje bajo por piloto</t>
-  </si>
-  <si>
-    <t>TDSYSTEM</t>
-  </si>
-  <si>
-    <t>Me contacto con el administrado por medio de llamada, indica que se va de vacaciones dos semanas y que el bajo marcaje es por una renuencia de los colaboradores, adicional quieren validar temas de vaciones regresando, no se arma aún reunión. 31/07/26</t>
-  </si>
-  <si>
-    <t>GRUPO JULIO</t>
-  </si>
-  <si>
-    <t>Tickets resueltos. Son por desconexión de reloj, pero pasa por bajas de voltaje en sus sucursales</t>
-  </si>
-  <si>
-    <t>DISTRIBUIDORA JUGUETRON</t>
-  </si>
-  <si>
-    <t>Reunión por NPS ok</t>
-  </si>
-  <si>
-    <t>IPS</t>
-  </si>
-  <si>
-    <t>No ha habido respuesta</t>
-  </si>
-  <si>
-    <t>Marcaje 27%</t>
-  </si>
-  <si>
-    <t>NSF DE MEXICO</t>
-  </si>
-  <si>
-    <t>Sin contacto</t>
-  </si>
-  <si>
-    <t>Marcaje 34%</t>
-  </si>
-  <si>
-    <t>Fletes Leal</t>
-  </si>
-  <si>
-    <t>Ver si además bajo marcaje sirve para vender alertas/ Tuve llamada con esta empresa, el marcaje bajo se debe a que sus coalaboradores no llegan a sitio donde se encuentra reloj para marcar y con Karla ya estan implementando APP, tendre reunión con ellos el día 14 de Agosto para dudas en plataforma.</t>
-  </si>
-  <si>
-    <t>Marcaje 50%</t>
-  </si>
-  <si>
-    <t>Marcaje 26% - NPS s/d - Tickets 0</t>
-  </si>
-  <si>
-    <t>HEXAGON MINING MEXICO</t>
-  </si>
-  <si>
-    <t>Implementación</t>
+    <t>Acompañamiento - Marcaje 11% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>29157-37879-36085-37826-36099-38471</t>
+  </si>
+  <si>
+    <t>J&amp;T EXPRESS CONEJO CORRIENDO R4 Central</t>
+  </si>
+  <si>
+    <t>Marcaje 50% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>J&amp;T EXPRESS CONEJO CORRIENDO Metropolitan</t>
+  </si>
+  <si>
+    <t>Marcaje 58% - NPS s/d - Tickets 0</t>
+  </si>
+  <si>
+    <t>CAPITAL BUS</t>
+  </si>
+  <si>
+    <t>Tenían temas de facturación, pero ya se está full en contacto y en vías de arreglo</t>
+  </si>
+  <si>
+    <t>Marcaje 93% - NPS 1 - Tickets 0</t>
+  </si>
+  <si>
+    <t>MANKA FOODS</t>
+  </si>
+  <si>
+    <t>Marcaje 82% - NPS s/d - Tickets 0. Variación ultimos 30 días de -54%</t>
   </si>
   <si>
     <t>Fecha</t>
@@ -418,12 +514,6 @@
   </si>
   <si>
     <t>Tenemos reunión el lunes 27 para validar planifiacion y temas en plataforma.</t>
-  </si>
-  <si>
-    <t>INTEGRITY PROTECTION SERVICES (IPS)</t>
-  </si>
-  <si>
-    <t>CAPITAL BUS</t>
   </si>
   <si>
     <t>Se contacta a segundo administrador por telefono 16/07/26, indica que marcan por CALL y que tienen problemas, en espera de que me den fecha para reu. Se manda mensaje de seguimiento sin respuesta (Lunes 20 y hoy 23)</t>
@@ -627,7 +717,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -675,6 +765,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
+    <xf numFmtId="9" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -977,7 +1068,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R163"/>
+  <dimension ref="A1:U152"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1269,73 +1360,76 @@
       <c r="H11" s="27"/>
     </row>
     <row r="12" spans="1:10">
-      <c r="A12" s="3"/>
-      <c r="B12" s="2">
-        <v>29825</v>
-      </c>
-      <c r="C12" s="2" t="s">
+      <c r="A12" s="16">
+        <v>46226</v>
+      </c>
+      <c r="B12" s="15">
+        <v>20172</v>
+      </c>
+      <c r="C12" s="15" t="s">
         <v>37</v>
       </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2" t="s">
+      <c r="D12" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="F12" s="15" t="s">
         <v>36</v>
       </c>
-      <c r="G12" s="2" t="s">
+      <c r="G12" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="H12" s="17"/>
+    </row>
+    <row r="13" spans="1:10">
+      <c r="A13" s="13">
+        <v>46226</v>
+      </c>
+      <c r="B13" s="9">
+        <v>23418</v>
+      </c>
+      <c r="C13" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="D13" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F13" s="9" t="s">
+        <v>36</v>
+      </c>
+      <c r="G13" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="H12" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10">
-      <c r="A13" s="16">
+      <c r="H13" s="14" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="7">
         <v>46226</v>
       </c>
-      <c r="B13" s="15">
-        <v>20172</v>
-      </c>
-      <c r="C13" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="F13" s="15" t="s">
+      <c r="B14" s="2">
+        <v>21190</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F14" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="G13" s="15" t="s">
+      <c r="G14" s="2" t="s">
         <v>36</v>
-      </c>
-      <c r="H13" s="17"/>
-    </row>
-    <row r="14" spans="1:10">
-      <c r="A14" s="13">
-        <v>46226</v>
-      </c>
-      <c r="B14" s="9">
-        <v>23418</v>
-      </c>
-      <c r="C14" s="9" t="s">
-        <v>41</v>
-      </c>
-      <c r="D14" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E14" s="9" t="s">
-        <v>42</v>
-      </c>
-      <c r="F14" s="9" t="s">
-        <v>36</v>
-      </c>
-      <c r="G14" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="H14" s="14" t="s">
-        <v>43</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -1343,7 +1437,7 @@
         <v>46226</v>
       </c>
       <c r="B15" s="2">
-        <v>21190</v>
+        <v>21657</v>
       </c>
       <c r="C15" s="2" t="s">
         <v>44</v>
@@ -1366,7 +1460,7 @@
         <v>46226</v>
       </c>
       <c r="B16" s="2">
-        <v>21657</v>
+        <v>6975</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>46</v>
@@ -1375,7 +1469,7 @@
         <v>15</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="F16" s="2" t="s">
         <v>36</v>
@@ -1384,21 +1478,21 @@
         <v>36</v>
       </c>
     </row>
-    <row r="17" spans="1:18">
+    <row r="17" spans="1:21">
       <c r="A17" s="7">
         <v>46226</v>
       </c>
       <c r="B17" s="2">
-        <v>6975</v>
+        <v>33503</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>15</v>
       </c>
       <c r="E17" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F17" s="2" t="s">
         <v>36</v>
@@ -1407,152 +1501,155 @@
         <v>36</v>
       </c>
     </row>
-    <row r="18" spans="1:18">
-      <c r="A18" s="7">
-        <v>46226</v>
-      </c>
-      <c r="B18" s="2">
-        <v>33503</v>
-      </c>
-      <c r="C18" s="2" t="s">
+    <row r="18" spans="1:21">
+      <c r="A18" s="28"/>
+      <c r="B18" s="25">
+        <v>32684</v>
+      </c>
+      <c r="C18" s="25" t="s">
         <v>49</v>
       </c>
-      <c r="D18" s="2" t="s">
+      <c r="D18" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="F18" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="G18" s="25" t="s">
+        <v>13</v>
+      </c>
+      <c r="H18" s="27"/>
+    </row>
+    <row r="19" spans="1:21" s="14" customFormat="1">
+      <c r="A19" s="20"/>
+      <c r="B19" s="9">
+        <v>24043</v>
+      </c>
+      <c r="C19" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G18" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19" spans="1:18">
-      <c r="A19" s="28"/>
-      <c r="B19" s="25">
-        <v>32684</v>
-      </c>
-      <c r="C19" s="25" t="s">
+      <c r="D19" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="E19" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="D19" s="25" t="s">
+      <c r="F19" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="G19" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="H19" s="38">
+        <v>0.33</v>
+      </c>
+      <c r="R19" s="32"/>
+    </row>
+    <row r="20" spans="1:21">
+      <c r="A20" s="3"/>
+      <c r="B20" s="2">
+        <v>28896</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D20" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E19" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="F19" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="G19" s="25" t="s">
-        <v>13</v>
-      </c>
-      <c r="H19" s="27"/>
-    </row>
-    <row r="20" spans="1:18" s="14" customFormat="1">
-      <c r="A20" s="20"/>
-      <c r="B20" s="9">
-        <v>24043</v>
-      </c>
-      <c r="C20" s="9" t="s">
-        <v>52</v>
-      </c>
-      <c r="D20" s="9" t="s">
+      <c r="E20" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G20" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H20" s="29">
+        <v>0.05</v>
+      </c>
+      <c r="R20" s="8"/>
+    </row>
+    <row r="21" spans="1:21" s="36" customFormat="1">
+      <c r="A21" s="34"/>
+      <c r="B21" s="33">
+        <v>31808</v>
+      </c>
+      <c r="C21" s="33" t="s">
+        <v>54</v>
+      </c>
+      <c r="D21" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="E20" s="9" t="s">
-        <v>53</v>
-      </c>
-      <c r="F20" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="G20" s="9" t="s">
+      <c r="E21" s="33" t="s">
+        <v>55</v>
+      </c>
+      <c r="F21" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="G21" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="H20" s="38">
-        <v>0.33</v>
-      </c>
-      <c r="R20" s="32"/>
-    </row>
-    <row r="21" spans="1:18">
-      <c r="A21" s="3"/>
-      <c r="B21" s="2">
-        <v>28896</v>
-      </c>
-      <c r="C21" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="D21" s="2" t="s">
+      <c r="H21" s="35">
+        <v>0.25</v>
+      </c>
+      <c r="R21" s="37"/>
+    </row>
+    <row r="22" spans="1:21">
+      <c r="A22" s="3"/>
+      <c r="B22" s="2">
+        <v>26920</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>56</v>
+      </c>
+      <c r="D22" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E21" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="F21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G21" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H21" s="29">
-        <v>0.05</v>
-      </c>
-      <c r="R21" s="8"/>
-    </row>
-    <row r="22" spans="1:18" s="36" customFormat="1">
-      <c r="A22" s="34"/>
-      <c r="B22" s="33">
-        <v>31808</v>
-      </c>
-      <c r="C22" s="33" t="s">
-        <v>56</v>
-      </c>
-      <c r="D22" s="33" t="s">
+      <c r="E22" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="F22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G22" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="R22" s="8"/>
+    </row>
+    <row r="23" spans="1:21" s="36" customFormat="1">
+      <c r="A23" s="34"/>
+      <c r="B23" s="33">
+        <v>2418</v>
+      </c>
+      <c r="C23" s="33" t="s">
+        <v>58</v>
+      </c>
+      <c r="D23" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="E22" s="33" t="s">
-        <v>57</v>
-      </c>
-      <c r="F22" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="G22" s="33" t="s">
+      <c r="E23" s="33" t="s">
+        <v>59</v>
+      </c>
+      <c r="F23" s="33" t="s">
+        <v>13</v>
+      </c>
+      <c r="G23" s="33" t="s">
         <v>17</v>
       </c>
-      <c r="H22" s="35">
-        <v>0.25</v>
-      </c>
-      <c r="R22" s="37"/>
-    </row>
-    <row r="23" spans="1:18">
-      <c r="A23" s="3"/>
-      <c r="B23" s="2">
-        <v>26920</v>
-      </c>
-      <c r="C23" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="D23" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E23" s="2" t="s">
-        <v>59</v>
-      </c>
-      <c r="F23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G23" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="R23" s="8"/>
-    </row>
-    <row r="24" spans="1:18" s="36" customFormat="1">
+      <c r="H23" s="35">
+        <v>0.52</v>
+      </c>
+      <c r="Q23" s="37"/>
+      <c r="R23" s="37"/>
+    </row>
+    <row r="24" spans="1:21" s="36" customFormat="1">
       <c r="A24" s="34"/>
       <c r="B24" s="33">
-        <v>2418</v>
+        <v>26371</v>
       </c>
       <c r="C24" s="33" t="s">
         <v>60</v>
@@ -1570,115 +1667,130 @@
         <v>17</v>
       </c>
       <c r="H24" s="35">
-        <v>0.52</v>
-      </c>
-      <c r="Q24" s="37"/>
+        <v>0.55000000000000004</v>
+      </c>
       <c r="R24" s="37"/>
     </row>
-    <row r="25" spans="1:18" s="36" customFormat="1">
-      <c r="A25" s="34"/>
-      <c r="B25" s="33">
-        <v>26371</v>
-      </c>
-      <c r="C25" s="33" t="s">
+    <row r="25" spans="1:21">
+      <c r="A25" s="3"/>
+      <c r="B25" s="2">
+        <v>21436</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="D25" s="33" t="s">
+      <c r="D25" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E25" s="33" t="s">
+      <c r="E25" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F25" s="33" t="s">
-        <v>13</v>
-      </c>
-      <c r="G25" s="33" t="s">
-        <v>17</v>
-      </c>
-      <c r="H25" s="35">
-        <v>0.55000000000000004</v>
-      </c>
-      <c r="R25" s="37"/>
-    </row>
-    <row r="26" spans="1:18">
-      <c r="A26" s="3"/>
-      <c r="B26" s="2">
-        <v>21436</v>
-      </c>
-      <c r="C26" s="2" t="s">
+      <c r="F25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="Q25" s="8"/>
+      <c r="R25" s="8"/>
+    </row>
+    <row r="26" spans="1:21">
+      <c r="A26" s="22" t="s">
         <v>64</v>
       </c>
-      <c r="D26" s="2" t="s">
+      <c r="B26" s="21">
+        <v>5725</v>
+      </c>
+      <c r="C26" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="D26" s="21"/>
+      <c r="E26" s="21" t="s">
+        <v>66</v>
+      </c>
+      <c r="F26" s="21" t="s">
+        <v>13</v>
+      </c>
+      <c r="G26" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="H26" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="I26" s="23">
+        <v>187</v>
+      </c>
+      <c r="J26" s="23">
+        <v>239</v>
+      </c>
+      <c r="K26" s="23"/>
+      <c r="L26" s="23"/>
+      <c r="M26" s="23"/>
+      <c r="N26" s="23"/>
+      <c r="O26" s="23"/>
+      <c r="P26" s="23"/>
+      <c r="Q26" s="23"/>
+      <c r="R26" s="23"/>
+      <c r="S26" s="23"/>
+      <c r="T26" s="23"/>
+      <c r="U26" s="23"/>
+    </row>
+    <row r="27" spans="1:21">
+      <c r="A27" s="3"/>
+      <c r="B27" s="2">
+        <v>25626</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="D27" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E26" s="2" t="s">
-        <v>65</v>
-      </c>
-      <c r="F26" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G26" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="Q26" s="8"/>
-      <c r="R26" s="8"/>
-    </row>
-    <row r="27" spans="1:18">
-      <c r="A27" s="22"/>
-      <c r="B27" s="21">
-        <v>5725</v>
-      </c>
-      <c r="C27" s="21" t="s">
-        <v>66</v>
-      </c>
-      <c r="D27" s="21"/>
-      <c r="E27" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="F27" s="21" t="s">
-        <v>13</v>
-      </c>
-      <c r="G27" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="H27" s="23" t="s">
+      <c r="E27" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H27" t="s">
         <v>31</v>
       </c>
+      <c r="Q27" s="8"/>
       <c r="R27" s="8"/>
     </row>
-    <row r="28" spans="1:18">
-      <c r="A28" s="3"/>
-      <c r="B28" s="2">
-        <v>25626</v>
-      </c>
-      <c r="C28" s="2" t="s">
-        <v>69</v>
-      </c>
-      <c r="D28" s="2" t="s">
+    <row r="28" spans="1:21">
+      <c r="A28" s="28"/>
+      <c r="B28" s="25">
+        <v>20338</v>
+      </c>
+      <c r="C28" s="25" t="s">
+        <v>71</v>
+      </c>
+      <c r="D28" s="25" t="s">
         <v>15</v>
       </c>
-      <c r="E28" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F28" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G28" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H28" t="s">
-        <v>31</v>
-      </c>
-      <c r="Q28" s="8"/>
+      <c r="E28" s="25" t="s">
+        <v>35</v>
+      </c>
+      <c r="F28" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="G28" s="25" t="s">
+        <v>72</v>
+      </c>
+      <c r="H28" s="27"/>
       <c r="R28" s="8"/>
     </row>
-    <row r="29" spans="1:18">
+    <row r="29" spans="1:21">
       <c r="A29" s="28"/>
       <c r="B29" s="25">
-        <v>20338</v>
+        <v>6055</v>
       </c>
       <c r="C29" s="25" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D29" s="25" t="s">
         <v>15</v>
@@ -1695,384 +1807,650 @@
       <c r="H29" s="27"/>
       <c r="R29" s="8"/>
     </row>
-    <row r="30" spans="1:18" s="36" customFormat="1">
-      <c r="A30" s="34"/>
-      <c r="B30" s="33">
-        <v>24372</v>
-      </c>
-      <c r="C30" s="33" t="s">
-        <v>73</v>
-      </c>
-      <c r="D30" s="33"/>
-      <c r="E30" s="33"/>
-      <c r="F30" s="33" t="s">
+    <row r="30" spans="1:21">
+      <c r="A30" s="18"/>
+      <c r="B30" s="15">
+        <v>21105</v>
+      </c>
+      <c r="C30" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="D30" s="15"/>
+      <c r="E30" s="15" t="s">
+        <v>75</v>
+      </c>
+      <c r="F30" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="G30" s="33" t="s">
+      <c r="G30" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="H30" s="36" t="s">
-        <v>74</v>
-      </c>
-      <c r="Q30" s="37"/>
-      <c r="R30" s="37"/>
-    </row>
-    <row r="31" spans="1:18">
-      <c r="A31" s="28"/>
-      <c r="B31" s="25">
-        <v>6055</v>
-      </c>
-      <c r="C31" s="25" t="s">
-        <v>75</v>
-      </c>
-      <c r="D31" s="25" t="s">
+      <c r="H30" s="39">
+        <v>0.44</v>
+      </c>
+      <c r="R30" s="8"/>
+    </row>
+    <row r="31" spans="1:21">
+      <c r="A31" s="18"/>
+      <c r="B31" s="15">
+        <v>18595</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>76</v>
+      </c>
+      <c r="D31" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E31" s="15" t="s">
+        <v>77</v>
+      </c>
+      <c r="F31" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="G31" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="H31" s="17"/>
+      <c r="Q31" s="8"/>
+      <c r="R31" s="8"/>
+    </row>
+    <row r="32" spans="1:21" s="14" customFormat="1">
+      <c r="A32" s="20"/>
+      <c r="B32" s="9">
+        <v>24950</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="D32" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="E31" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="F31" s="25" t="s">
+      <c r="E32" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="F32" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="G31" s="25" t="s">
+      <c r="G32" s="9" t="s">
+        <v>17</v>
+      </c>
+      <c r="Q32" s="32"/>
+      <c r="R32" s="32"/>
+    </row>
+    <row r="33" spans="1:18">
+      <c r="A33" s="18"/>
+      <c r="B33" s="15">
+        <v>30644</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>80</v>
+      </c>
+      <c r="D33" s="15" t="s">
+        <v>11</v>
+      </c>
+      <c r="E33" s="15" t="s">
+        <v>81</v>
+      </c>
+      <c r="F33" s="15" t="s">
         <v>72</v>
       </c>
-      <c r="H31" s="27"/>
-      <c r="R31" s="8"/>
-    </row>
-    <row r="32" spans="1:18">
-      <c r="A32" s="3"/>
-      <c r="B32" s="2">
-        <v>6588</v>
-      </c>
-      <c r="C32" s="2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G32" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="H32" s="29">
-        <v>0.42</v>
-      </c>
-      <c r="Q32" s="8"/>
-      <c r="R32" s="8"/>
-    </row>
-    <row r="33" spans="1:18">
-      <c r="A33" s="3"/>
-      <c r="B33" s="2">
-        <v>21105</v>
-      </c>
-      <c r="C33" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="G33" s="2" t="s">
+      <c r="G33" s="15" t="s">
         <v>17</v>
       </c>
-      <c r="H33" s="29">
-        <v>0.44</v>
-      </c>
+      <c r="H33" s="17"/>
       <c r="R33" s="8"/>
     </row>
     <row r="34" spans="1:18">
       <c r="A34" s="18"/>
       <c r="B34" s="15">
-        <v>18595</v>
+        <v>24336</v>
       </c>
       <c r="C34" s="15" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="D34" s="15" t="s">
         <v>11</v>
       </c>
       <c r="E34" s="15" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="F34" s="15" t="s">
         <v>72</v>
       </c>
       <c r="G34" s="15" t="s">
-        <v>72</v>
+        <v>17</v>
       </c>
       <c r="H34" s="17"/>
       <c r="Q34" s="8"/>
       <c r="R34" s="8"/>
     </row>
-    <row r="35" spans="1:18" s="14" customFormat="1">
-      <c r="A35" s="20"/>
-      <c r="B35" s="9">
-        <v>24950</v>
-      </c>
-      <c r="C35" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D35" s="9" t="s">
+    <row r="35" spans="1:18">
+      <c r="A35" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B35" s="2">
+        <v>30029</v>
+      </c>
+      <c r="C35" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2" t="s">
+        <v>86</v>
+      </c>
+      <c r="F35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G35" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H35" t="s">
+        <v>87</v>
+      </c>
+      <c r="I35">
+        <v>250</v>
+      </c>
+      <c r="J35">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="36" spans="1:18">
+      <c r="A36" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B36" s="2">
+        <v>33301</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>88</v>
+      </c>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="F36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G36" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H36" t="s">
+        <v>90</v>
+      </c>
+      <c r="I36">
+        <v>165</v>
+      </c>
+      <c r="J36">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="37" spans="1:18">
+      <c r="A37" s="3"/>
+      <c r="B37" s="2">
+        <v>20442</v>
+      </c>
+      <c r="C37" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D37" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E35" s="9" t="s">
-        <v>81</v>
-      </c>
-      <c r="F35" s="9" t="s">
+      <c r="E37" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="F37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G37" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H37" t="s">
+        <v>93</v>
+      </c>
+      <c r="R37" s="8"/>
+    </row>
+    <row r="38" spans="1:18">
+      <c r="B38" s="2"/>
+      <c r="C38" s="2" t="s">
+        <v>94</v>
+      </c>
+      <c r="D38" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H38" s="3" t="s">
+        <v>95</v>
+      </c>
+      <c r="K38">
+        <v>188</v>
+      </c>
+      <c r="L38">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="39" spans="1:18">
+      <c r="A39" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="B39" s="2">
+        <v>6588</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D39" s="2"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G35" s="9" t="s">
-        <v>17</v>
-      </c>
-      <c r="Q35" s="32"/>
-      <c r="R35" s="32"/>
-    </row>
-    <row r="36" spans="1:18">
-      <c r="A36" s="18"/>
-      <c r="B36" s="15">
-        <v>30644</v>
-      </c>
-      <c r="C36" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="D36" s="15" t="s">
+      <c r="G39" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H39" t="s">
+        <v>98</v>
+      </c>
+      <c r="I39">
+        <v>1826</v>
+      </c>
+      <c r="J39">
+        <v>1416</v>
+      </c>
+    </row>
+    <row r="40" spans="1:18">
+      <c r="A40" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B40" s="2">
+        <v>26081</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="E36" s="15" t="s">
-        <v>83</v>
-      </c>
-      <c r="F36" s="15" t="s">
+      <c r="E40" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F40" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G36" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="H36" s="17"/>
-      <c r="R36" s="8"/>
-    </row>
-    <row r="37" spans="1:18">
-      <c r="A37" s="18"/>
-      <c r="B37" s="15">
-        <v>24336</v>
-      </c>
-      <c r="C37" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="D37" s="15" t="s">
-        <v>11</v>
-      </c>
-      <c r="E37" s="15" t="s">
-        <v>85</v>
-      </c>
-      <c r="F37" s="15" t="s">
+      <c r="G40" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="G37" s="15" t="s">
-        <v>17</v>
-      </c>
-      <c r="H37" s="17"/>
-      <c r="Q37" s="8"/>
-      <c r="R37" s="8"/>
-    </row>
-    <row r="38" spans="1:18">
-      <c r="A38" s="3"/>
-      <c r="B38" s="2">
-        <v>30029</v>
-      </c>
-      <c r="C38" s="2" t="s">
-        <v>86</v>
-      </c>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F38" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G38" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="H38" t="s">
-        <v>88</v>
-      </c>
-      <c r="R38" s="8"/>
-    </row>
-    <row r="39" spans="1:18">
-      <c r="A39" s="3"/>
-      <c r="B39" s="2">
-        <v>33301</v>
-      </c>
-      <c r="C39" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="D39" s="2"/>
-      <c r="E39" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="F39" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G39" s="2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H39" t="s">
-        <v>91</v>
-      </c>
-      <c r="R39" s="8"/>
-    </row>
-    <row r="40" spans="1:18">
-      <c r="A40" s="3"/>
-      <c r="B40" s="2">
-        <v>20442</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>92</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="E40" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F40" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="G40" s="2" t="s">
-        <v>13</v>
-      </c>
       <c r="H40" t="s">
-        <v>94</v>
-      </c>
-      <c r="R40" s="8"/>
+        <v>101</v>
+      </c>
+      <c r="I40">
+        <v>1396</v>
+      </c>
+      <c r="J40">
+        <v>985</v>
+      </c>
     </row>
     <row r="41" spans="1:18">
       <c r="A41" s="3" t="s">
-        <v>95</v>
-      </c>
-      <c r="B41" s="2"/>
+        <v>64</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>102</v>
+      </c>
       <c r="C41" s="2" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="D41" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="E41" s="2"/>
+        <v>15</v>
+      </c>
+      <c r="E41" s="2" t="s">
+        <v>19</v>
+      </c>
       <c r="F41" s="2" t="s">
-        <v>13</v>
+        <v>72</v>
       </c>
       <c r="G41" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="K41">
-        <v>188</v>
-      </c>
-      <c r="L41">
-        <v>73</v>
+        <v>72</v>
+      </c>
+      <c r="H41" t="s">
+        <v>104</v>
+      </c>
+      <c r="I41">
+        <v>762</v>
+      </c>
+      <c r="J41">
+        <v>147</v>
       </c>
     </row>
     <row r="42" spans="1:18">
-      <c r="A42" s="3"/>
-      <c r="B42" s="2"/>
-      <c r="C42" s="2"/>
+      <c r="A42" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B42" s="2">
+        <v>24372</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>105</v>
+      </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-      <c r="G42" s="2"/>
+      <c r="F42" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G42" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H42" t="s">
+        <v>106</v>
+      </c>
+      <c r="I42">
+        <v>33</v>
+      </c>
+      <c r="J42">
+        <v>357</v>
+      </c>
     </row>
     <row r="43" spans="1:18">
-      <c r="A43" s="3"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
+      <c r="A43" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B43" s="2">
+        <v>22923</v>
+      </c>
+      <c r="C43" s="2" t="s">
+        <v>107</v>
+      </c>
       <c r="D43" s="2"/>
       <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-      <c r="G43" s="2"/>
+      <c r="F43" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="G43" s="2" t="s">
+        <v>72</v>
+      </c>
+      <c r="H43" t="s">
+        <v>108</v>
+      </c>
+      <c r="I43">
+        <v>0</v>
+      </c>
+      <c r="J43">
+        <v>740</v>
+      </c>
     </row>
     <row r="44" spans="1:18">
-      <c r="A44" s="3"/>
-      <c r="B44" s="2"/>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-      <c r="G44" s="2"/>
+      <c r="A44" s="3" t="s">
+        <v>109</v>
+      </c>
+      <c r="B44" s="2">
+        <v>26102</v>
+      </c>
+      <c r="C44" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="D44" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="F44" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G44" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H44" t="s">
+        <v>111</v>
+      </c>
+      <c r="I44">
+        <v>1549</v>
+      </c>
+      <c r="J44">
+        <v>430</v>
+      </c>
     </row>
     <row r="45" spans="1:18">
-      <c r="A45" s="3"/>
-      <c r="B45" s="2"/>
-      <c r="C45" s="2"/>
+      <c r="A45" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B45" s="2">
+        <v>23879</v>
+      </c>
+      <c r="C45" s="2" t="s">
+        <v>112</v>
+      </c>
       <c r="D45" s="2"/>
       <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-      <c r="G45" s="2"/>
+      <c r="F45" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G45" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H45" t="s">
+        <v>113</v>
+      </c>
+      <c r="I45">
+        <v>414</v>
+      </c>
+      <c r="J45">
+        <v>177</v>
+      </c>
     </row>
     <row r="46" spans="1:18">
-      <c r="A46" s="3"/>
-      <c r="B46" s="2"/>
-      <c r="C46" s="2"/>
+      <c r="A46" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B46" s="2">
+        <v>21914</v>
+      </c>
+      <c r="C46" s="2" t="s">
+        <v>114</v>
+      </c>
       <c r="D46" s="2"/>
       <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-      <c r="G46" s="2"/>
+      <c r="F46" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G46" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H46" t="s">
+        <v>115</v>
+      </c>
+      <c r="I46">
+        <v>408</v>
+      </c>
+      <c r="J46">
+        <v>181</v>
+      </c>
     </row>
     <row r="47" spans="1:18">
-      <c r="A47" s="3"/>
-      <c r="B47" s="2"/>
-      <c r="C47" s="2"/>
+      <c r="A47" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B47" s="2">
+        <v>24310</v>
+      </c>
+      <c r="C47" s="2" t="s">
+        <v>116</v>
+      </c>
       <c r="D47" s="2"/>
       <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-      <c r="G47" s="2"/>
+      <c r="F47" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G47" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H47" t="s">
+        <v>117</v>
+      </c>
+      <c r="I47">
+        <v>249</v>
+      </c>
+      <c r="J47">
+        <v>107</v>
+      </c>
     </row>
     <row r="48" spans="1:18">
-      <c r="A48" s="3"/>
-      <c r="B48" s="2"/>
-      <c r="C48" s="2"/>
+      <c r="A48" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="B48" s="2">
+        <v>29825</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>118</v>
+      </c>
       <c r="D48" s="2"/>
       <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-      <c r="G48" s="2"/>
-    </row>
-    <row r="49" spans="1:7">
-      <c r="A49" s="3"/>
-      <c r="B49" s="2"/>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-      <c r="G49" s="2"/>
-    </row>
-    <row r="50" spans="1:7">
-      <c r="A50" s="3"/>
-      <c r="B50" s="2"/>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-      <c r="G50" s="2"/>
-    </row>
-    <row r="51" spans="1:7">
-      <c r="A51" s="3"/>
+      <c r="F48" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G48" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H48" t="s">
+        <v>119</v>
+      </c>
+      <c r="I48">
+        <v>212</v>
+      </c>
+      <c r="J48">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10">
+      <c r="A49" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B49" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C49" s="2" t="s">
+        <v>121</v>
+      </c>
+      <c r="D49" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E49" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F49" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G49" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H49" t="s">
+        <v>122</v>
+      </c>
+      <c r="I49">
+        <v>0</v>
+      </c>
+      <c r="J49">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10">
+      <c r="A50" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B50" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="D50" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="E50" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="F50" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G50" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="H50" t="s">
+        <v>124</v>
+      </c>
+      <c r="I50">
+        <v>0</v>
+      </c>
+      <c r="J50">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10">
+      <c r="A51" s="3" t="s">
+        <v>96</v>
+      </c>
       <c r="B51" s="2"/>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-      <c r="G51" s="2"/>
-    </row>
-    <row r="52" spans="1:7">
-      <c r="A52" s="3"/>
-      <c r="B52" s="2"/>
-      <c r="C52" s="2"/>
+      <c r="C51" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D51" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="E51" s="2" t="s">
+        <v>126</v>
+      </c>
+      <c r="F51" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G51" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H51" t="s">
+        <v>127</v>
+      </c>
+      <c r="I51">
+        <v>330</v>
+      </c>
+      <c r="J51">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10">
+      <c r="A52" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="B52" s="2">
+        <v>18457</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>128</v>
+      </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-      <c r="G52" s="2"/>
-    </row>
-    <row r="53" spans="1:7">
+      <c r="F52" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="G52" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H52" t="s">
+        <v>129</v>
+      </c>
+      <c r="I52">
+        <v>156</v>
+      </c>
+      <c r="J52">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10">
       <c r="A53" s="3"/>
       <c r="B53" s="2"/>
       <c r="C53" s="2"/>
@@ -2081,7 +2459,7 @@
       <c r="F53" s="2"/>
       <c r="G53" s="2"/>
     </row>
-    <row r="54" spans="1:7">
+    <row r="54" spans="1:10">
       <c r="A54" s="3"/>
       <c r="B54" s="2"/>
       <c r="C54" s="2"/>
@@ -2090,7 +2468,7 @@
       <c r="F54" s="2"/>
       <c r="G54" s="2"/>
     </row>
-    <row r="55" spans="1:7">
+    <row r="55" spans="1:10">
       <c r="A55" s="3"/>
       <c r="B55" s="2"/>
       <c r="C55" s="2"/>
@@ -2099,7 +2477,7 @@
       <c r="F55" s="2"/>
       <c r="G55" s="2"/>
     </row>
-    <row r="56" spans="1:7">
+    <row r="56" spans="1:10">
       <c r="A56" s="3"/>
       <c r="B56" s="2"/>
       <c r="C56" s="2"/>
@@ -2108,7 +2486,7 @@
       <c r="F56" s="2"/>
       <c r="G56" s="2"/>
     </row>
-    <row r="57" spans="1:7">
+    <row r="57" spans="1:10">
       <c r="A57" s="3"/>
       <c r="B57" s="2"/>
       <c r="C57" s="2"/>
@@ -2117,7 +2495,7 @@
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
     </row>
-    <row r="58" spans="1:7">
+    <row r="58" spans="1:10">
       <c r="A58" s="3"/>
       <c r="B58" s="2"/>
       <c r="C58" s="2"/>
@@ -2126,7 +2504,7 @@
       <c r="F58" s="2"/>
       <c r="G58" s="2"/>
     </row>
-    <row r="59" spans="1:7">
+    <row r="59" spans="1:10">
       <c r="A59" s="3"/>
       <c r="B59" s="2"/>
       <c r="C59" s="2"/>
@@ -2135,7 +2513,7 @@
       <c r="F59" s="2"/>
       <c r="G59" s="2"/>
     </row>
-    <row r="60" spans="1:7">
+    <row r="60" spans="1:10">
       <c r="A60" s="3"/>
       <c r="B60" s="2"/>
       <c r="C60" s="2"/>
@@ -2144,7 +2522,7 @@
       <c r="F60" s="2"/>
       <c r="G60" s="2"/>
     </row>
-    <row r="61" spans="1:7">
+    <row r="61" spans="1:10">
       <c r="A61" s="3"/>
       <c r="B61" s="2"/>
       <c r="C61" s="2"/>
@@ -2153,7 +2531,7 @@
       <c r="F61" s="2"/>
       <c r="G61" s="2"/>
     </row>
-    <row r="62" spans="1:7">
+    <row r="62" spans="1:10">
       <c r="A62" s="3"/>
       <c r="B62" s="2"/>
       <c r="C62" s="2"/>
@@ -2162,7 +2540,7 @@
       <c r="F62" s="2"/>
       <c r="G62" s="2"/>
     </row>
-    <row r="63" spans="1:7">
+    <row r="63" spans="1:10">
       <c r="A63" s="3"/>
       <c r="B63" s="2"/>
       <c r="C63" s="2"/>
@@ -2171,7 +2549,7 @@
       <c r="F63" s="2"/>
       <c r="G63" s="2"/>
     </row>
-    <row r="64" spans="1:7">
+    <row r="64" spans="1:10">
       <c r="A64" s="3"/>
       <c r="B64" s="2"/>
       <c r="C64" s="2"/>
@@ -2972,109 +3350,10 @@
       <c r="F152" s="2"/>
       <c r="G152" s="2"/>
     </row>
-    <row r="153" spans="1:7">
-      <c r="A153" s="3"/>
-      <c r="B153" s="2"/>
-      <c r="C153" s="2"/>
-      <c r="D153" s="2"/>
-      <c r="E153" s="2"/>
-      <c r="F153" s="2"/>
-      <c r="G153" s="2"/>
-    </row>
-    <row r="154" spans="1:7">
-      <c r="A154" s="3"/>
-      <c r="B154" s="2"/>
-      <c r="C154" s="2"/>
-      <c r="D154" s="2"/>
-      <c r="E154" s="2"/>
-      <c r="F154" s="2"/>
-      <c r="G154" s="2"/>
-    </row>
-    <row r="155" spans="1:7">
-      <c r="A155" s="3"/>
-      <c r="B155" s="2"/>
-      <c r="C155" s="2"/>
-      <c r="D155" s="2"/>
-      <c r="E155" s="2"/>
-      <c r="F155" s="2"/>
-      <c r="G155" s="2"/>
-    </row>
-    <row r="156" spans="1:7">
-      <c r="A156" s="3"/>
-      <c r="B156" s="2"/>
-      <c r="C156" s="2"/>
-      <c r="D156" s="2"/>
-      <c r="E156" s="2"/>
-      <c r="F156" s="2"/>
-      <c r="G156" s="2"/>
-    </row>
-    <row r="157" spans="1:7">
-      <c r="A157" s="3"/>
-      <c r="B157" s="2"/>
-      <c r="C157" s="2"/>
-      <c r="D157" s="2"/>
-      <c r="E157" s="2"/>
-      <c r="F157" s="2"/>
-      <c r="G157" s="2"/>
-    </row>
-    <row r="158" spans="1:7">
-      <c r="A158" s="3"/>
-      <c r="B158" s="2"/>
-      <c r="C158" s="2"/>
-      <c r="D158" s="2"/>
-      <c r="E158" s="2"/>
-      <c r="F158" s="2"/>
-      <c r="G158" s="2"/>
-    </row>
-    <row r="159" spans="1:7">
-      <c r="A159" s="3"/>
-      <c r="B159" s="2"/>
-      <c r="C159" s="2"/>
-      <c r="D159" s="2"/>
-      <c r="E159" s="2"/>
-      <c r="F159" s="2"/>
-      <c r="G159" s="2"/>
-    </row>
-    <row r="160" spans="1:7">
-      <c r="A160" s="3"/>
-      <c r="B160" s="2"/>
-      <c r="C160" s="2"/>
-      <c r="D160" s="2"/>
-      <c r="E160" s="2"/>
-      <c r="F160" s="2"/>
-      <c r="G160" s="2"/>
-    </row>
-    <row r="161" spans="1:7">
-      <c r="A161" s="3"/>
-      <c r="B161" s="2"/>
-      <c r="C161" s="2"/>
-      <c r="D161" s="2"/>
-      <c r="E161" s="2"/>
-      <c r="F161" s="2"/>
-      <c r="G161" s="2"/>
-    </row>
-    <row r="162" spans="1:7">
-      <c r="A162" s="3"/>
-      <c r="B162" s="2"/>
-      <c r="C162" s="2"/>
-      <c r="D162" s="2"/>
-      <c r="E162" s="2"/>
-      <c r="F162" s="2"/>
-      <c r="G162" s="2"/>
-    </row>
-    <row r="163" spans="1:7">
-      <c r="A163" s="3"/>
-      <c r="B163" s="2"/>
-      <c r="C163" s="2"/>
-      <c r="D163" s="2"/>
-      <c r="E163" s="2"/>
-      <c r="F163" s="2"/>
-      <c r="G163" s="2"/>
-    </row>
   </sheetData>
-  <autoFilter ref="B1:G40" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="B1:G37" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" errorTitle="Estado inválido" error="Elige &quot;Seguimiento&quot; o &quot;Resuelta&quot; de la lista." sqref="D2:D164 A2:A164" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Estado inválido" error="Elige &quot;Seguimiento&quot; o &quot;Resuelta&quot; de la lista." sqref="H38 A2:A37 D2:D153 A39:A153" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Seguimiento,Resuelta"</formula1>
     </dataValidation>
   </dataValidations>
@@ -3105,19 +3384,19 @@
         <v>6</v>
       </c>
       <c r="N8" t="s">
-        <v>98</v>
+        <v>130</v>
       </c>
       <c r="O8" t="s">
-        <v>99</v>
+        <v>131</v>
       </c>
       <c r="P8" t="s">
-        <v>100</v>
+        <v>132</v>
       </c>
       <c r="Q8" t="s">
         <v>8</v>
       </c>
       <c r="R8" t="s">
-        <v>101</v>
+        <v>133</v>
       </c>
     </row>
     <row r="9" spans="9:18">
@@ -3125,7 +3404,7 @@
         <v>2418</v>
       </c>
       <c r="J9" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="M9" t="s">
         <v>13</v>
@@ -3134,7 +3413,7 @@
         <v>46230</v>
       </c>
       <c r="P9" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q9">
         <v>89</v>
@@ -3145,7 +3424,7 @@
         <v>28896</v>
       </c>
       <c r="J10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="M10" t="s">
         <v>13</v>
@@ -3154,7 +3433,7 @@
         <v>46230</v>
       </c>
       <c r="P10" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q10">
         <v>109</v>
@@ -3174,7 +3453,7 @@
         <v>46230</v>
       </c>
       <c r="P11" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q11">
         <v>117</v>
@@ -3185,7 +3464,7 @@
         <v>26371</v>
       </c>
       <c r="J12" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="M12" t="s">
         <v>13</v>
@@ -3194,7 +3473,7 @@
         <v>46230</v>
       </c>
       <c r="P12" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q12">
         <v>140</v>
@@ -3205,7 +3484,7 @@
         <v>20442</v>
       </c>
       <c r="J13" t="s">
-        <v>103</v>
+        <v>135</v>
       </c>
       <c r="M13" t="s">
         <v>13</v>
@@ -3214,7 +3493,7 @@
         <v>46230</v>
       </c>
       <c r="P13" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q13">
         <v>161</v>
@@ -3243,7 +3522,7 @@
         <v>46230</v>
       </c>
       <c r="P14" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q14">
         <v>171</v>
@@ -3254,7 +3533,7 @@
         <v>26920</v>
       </c>
       <c r="J15" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="M15" t="s">
         <v>13</v>
@@ -3263,7 +3542,7 @@
         <v>46230</v>
       </c>
       <c r="P15" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q15">
         <v>188</v>
@@ -3292,7 +3571,7 @@
         <v>46230</v>
       </c>
       <c r="P16" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q16">
         <v>220</v>
@@ -3303,7 +3582,7 @@
         <v>24043</v>
       </c>
       <c r="J17" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="M17" t="s">
         <v>13</v>
@@ -3312,7 +3591,7 @@
         <v>46230</v>
       </c>
       <c r="P17" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q17">
         <v>273</v>
@@ -3323,7 +3602,7 @@
         <v>31808</v>
       </c>
       <c r="J18" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="M18" t="s">
         <v>13</v>
@@ -3332,7 +3611,7 @@
         <v>46230</v>
       </c>
       <c r="P18" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q18">
         <v>375</v>
@@ -3343,7 +3622,7 @@
         <v>21436</v>
       </c>
       <c r="J19" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="M19" t="s">
         <v>13</v>
@@ -3352,7 +3631,7 @@
         <v>46230</v>
       </c>
       <c r="P19" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q19">
         <v>435</v>
@@ -3363,7 +3642,7 @@
         <v>5725</v>
       </c>
       <c r="J20" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="M20" t="s">
         <v>13</v>
@@ -3372,7 +3651,7 @@
         <v>46230</v>
       </c>
       <c r="P20" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q20">
         <v>156</v>
@@ -3389,7 +3668,7 @@
         <v>15</v>
       </c>
       <c r="L21" t="s">
-        <v>104</v>
+        <v>136</v>
       </c>
       <c r="M21" t="s">
         <v>17</v>
@@ -3401,7 +3680,7 @@
         <v>46230</v>
       </c>
       <c r="P21" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q21">
         <v>156</v>
@@ -3412,7 +3691,7 @@
         <v>33301</v>
       </c>
       <c r="J22" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="M22" t="s">
         <v>13</v>
@@ -3421,7 +3700,7 @@
         <v>46230</v>
       </c>
       <c r="P22" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q22">
         <v>165</v>
@@ -3432,13 +3711,13 @@
         <v>32684</v>
       </c>
       <c r="J23" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="K23" t="s">
         <v>15</v>
       </c>
       <c r="L23" t="s">
-        <v>105</v>
+        <v>137</v>
       </c>
       <c r="M23" t="s">
         <v>13</v>
@@ -3447,7 +3726,7 @@
         <v>46230</v>
       </c>
       <c r="P23" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q23">
         <v>166</v>
@@ -3458,7 +3737,7 @@
         <v>36723</v>
       </c>
       <c r="J24" t="s">
-        <v>106</v>
+        <v>138</v>
       </c>
       <c r="M24" t="s">
         <v>13</v>
@@ -3467,7 +3746,7 @@
         <v>46230</v>
       </c>
       <c r="P24" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q24">
         <v>187</v>
@@ -3475,7 +3754,7 @@
     </row>
     <row r="25" spans="9:17">
       <c r="J25" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="M25" t="s">
         <v>13</v>
@@ -3484,7 +3763,7 @@
         <v>46230</v>
       </c>
       <c r="P25" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q25">
         <v>188</v>
@@ -3501,7 +3780,7 @@
         <v>15</v>
       </c>
       <c r="L26" t="s">
-        <v>107</v>
+        <v>139</v>
       </c>
       <c r="M26" t="s">
         <v>17</v>
@@ -3513,7 +3792,7 @@
         <v>46230</v>
       </c>
       <c r="P26" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q26">
         <v>189</v>
@@ -3524,7 +3803,7 @@
         <v>30029</v>
       </c>
       <c r="J27" t="s">
-        <v>108</v>
+        <v>85</v>
       </c>
       <c r="M27" t="s">
         <v>13</v>
@@ -3533,7 +3812,7 @@
         <v>46230</v>
       </c>
       <c r="P27" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q27">
         <v>270</v>
@@ -3559,7 +3838,7 @@
         <v>46230</v>
       </c>
       <c r="P28" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q28">
         <v>290</v>
@@ -3567,7 +3846,7 @@
     </row>
     <row r="29" spans="9:17">
       <c r="J29" t="s">
-        <v>109</v>
+        <v>125</v>
       </c>
       <c r="M29" t="s">
         <v>13</v>
@@ -3576,7 +3855,7 @@
         <v>46230</v>
       </c>
       <c r="P29" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q29">
         <v>303</v>
@@ -3605,7 +3884,7 @@
         <v>46230</v>
       </c>
       <c r="P30" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q30">
         <v>310</v>
@@ -3619,7 +3898,7 @@
         <v>15</v>
       </c>
       <c r="L31" t="s">
-        <v>110</v>
+        <v>140</v>
       </c>
       <c r="M31" t="s">
         <v>17</v>
@@ -3631,7 +3910,7 @@
         <v>46230</v>
       </c>
       <c r="P31" t="s">
-        <v>102</v>
+        <v>134</v>
       </c>
       <c r="Q31">
         <v>423</v>
@@ -3642,7 +3921,7 @@
         <v>27671</v>
       </c>
       <c r="J32" t="s">
-        <v>111</v>
+        <v>141</v>
       </c>
       <c r="M32" t="s">
         <v>13</v>
@@ -3651,7 +3930,7 @@
         <v>46230</v>
       </c>
       <c r="P32" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
       <c r="Q32">
         <v>160</v>
@@ -3668,7 +3947,7 @@
         <v>15</v>
       </c>
       <c r="L33" t="s">
-        <v>113</v>
+        <v>143</v>
       </c>
       <c r="M33" t="s">
         <v>13</v>
@@ -3680,7 +3959,7 @@
         <v>46230</v>
       </c>
       <c r="P33" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
       <c r="Q33">
         <v>223</v>
@@ -3691,7 +3970,7 @@
         <v>29844</v>
       </c>
       <c r="J34" t="s">
-        <v>114</v>
+        <v>144</v>
       </c>
       <c r="M34" t="s">
         <v>13</v>
@@ -3700,7 +3979,7 @@
         <v>46230</v>
       </c>
       <c r="P34" t="s">
-        <v>112</v>
+        <v>142</v>
       </c>
       <c r="Q34">
         <v>372</v>
@@ -3721,7 +4000,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="4" t="s">
-        <v>115</v>
+        <v>145</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -3729,12 +4008,12 @@
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="5" t="s">
-        <v>116</v>
+        <v>146</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="5" t="s">
-        <v>117</v>
+        <v>147</v>
       </c>
     </row>
     <row r="5" spans="1:1">
@@ -3742,37 +4021,37 @@
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="6" t="s">
-        <v>118</v>
+        <v>148</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="5" t="s">
-        <v>119</v>
+        <v>149</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="5" t="s">
-        <v>120</v>
+        <v>150</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="5" t="s">
-        <v>121</v>
+        <v>151</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="5" t="s">
-        <v>122</v>
+        <v>152</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="5" t="s">
-        <v>123</v>
+        <v>153</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="5" t="s">
-        <v>124</v>
+        <v>154</v>
       </c>
     </row>
     <row r="13" spans="1:1">
@@ -3780,27 +4059,27 @@
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="6" t="s">
-        <v>125</v>
+        <v>155</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="5" t="s">
-        <v>126</v>
+        <v>156</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="5" t="s">
-        <v>127</v>
+        <v>157</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="5" t="s">
-        <v>128</v>
+        <v>158</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="5" t="s">
-        <v>129</v>
+        <v>159</v>
       </c>
     </row>
     <row r="19" spans="1:1">
@@ -3808,12 +4087,12 @@
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="5" t="s">
-        <v>130</v>
+        <v>160</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="5" t="s">
-        <v>131</v>
+        <v>161</v>
       </c>
     </row>
   </sheetData>

</xml_diff>